<commit_message>
Research and List of Extension
</commit_message>
<xml_diff>
--- a/backend/utils/template2.xlsx
+++ b/backend/utils/template2.xlsx
@@ -8,15 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\My Stuff\Github\IPCR_GENERATOR-Thesis\backend\utils\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82BD64F3-E137-446E-8003-AA9CA0348EDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24C815B8-D821-4F73-A174-A65654E4106F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1st Quarter" sheetId="1" r:id="rId1"/>
     <sheet name="2nd Quarter" sheetId="9" r:id="rId2"/>
     <sheet name="3rd Quarter" sheetId="10" r:id="rId3"/>
     <sheet name="4th Quarter" sheetId="11" r:id="rId4"/>
+    <sheet name="RESEARCH" sheetId="13" r:id="rId5"/>
+    <sheet name="EXTENSION" sheetId="12" r:id="rId6"/>
+    <sheet name="LIST OF EXTENSIONS" sheetId="14" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,40 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="13">
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="13"/>
-        <color rgb="FF000000"/>
-        <rFont val="Poppins"/>
-      </rPr>
-      <t xml:space="preserve">COLLEGE OF COMPUTER STUDIES
-Santa Cruz Campus
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="13"/>
-        <color rgb="FF783F04"/>
-        <rFont val="Poppins"/>
-      </rPr>
-      <t>JANUARY TO MARCH 2025</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="13"/>
-        <color rgb="FF000000"/>
-        <rFont val="Poppins"/>
-      </rPr>
-      <t xml:space="preserve">
- FACULTY SEMINAR, CONFERENCE AND TRAINING
-</t>
-    </r>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="82">
   <si>
     <t>Title Training/Seminar/
  Conference</t>
@@ -182,6 +152,240 @@
 </t>
     </r>
   </si>
+  <si>
+    <t>CCS Extension and Services Target 2025 - Santa Cruz</t>
+  </si>
+  <si>
+    <t>2025 EXTENSION TARGET</t>
+  </si>
+  <si>
+    <t>COLLEGE</t>
+  </si>
+  <si>
+    <t>INDICATORS</t>
+  </si>
+  <si>
+    <t>1st Quarter</t>
+  </si>
+  <si>
+    <t>2nd Quarter</t>
+  </si>
+  <si>
+    <t>3rd Quarter</t>
+  </si>
+  <si>
+    <t>4th Quarter</t>
+  </si>
+  <si>
+    <t>Total Target</t>
+  </si>
+  <si>
+    <t>Total Accomplished</t>
+  </si>
+  <si>
+    <t>Target</t>
+  </si>
+  <si>
+    <t>Accomplishment</t>
+  </si>
+  <si>
+    <t>CCS</t>
+  </si>
+  <si>
+    <t>Number of Active Partnership</t>
+  </si>
+  <si>
+    <t>Number of Trainess</t>
+  </si>
+  <si>
+    <t>Number of Extension Program</t>
+  </si>
+  <si>
+    <t>Instructor Multiply by 1</t>
+  </si>
+  <si>
+    <t>Assistant Professor Multiply by 1.1</t>
+  </si>
+  <si>
+    <t>Associate Professor Multiply by 1.2</t>
+  </si>
+  <si>
+    <t>Q2</t>
+  </si>
+  <si>
+    <t>Q3</t>
+  </si>
+  <si>
+    <t>Q4</t>
+  </si>
+  <si>
+    <t>Instructor</t>
+  </si>
+  <si>
+    <t>Assistant Professor</t>
+  </si>
+  <si>
+    <t>Associate Professor</t>
+  </si>
+  <si>
+    <t>FACULTY LAST NAME</t>
+  </si>
+  <si>
+    <t>RANK</t>
+  </si>
+  <si>
+    <t>2nd Semester AY: 2024-2025</t>
+  </si>
+  <si>
+    <t>1st Semester AY: 2025-2026</t>
+  </si>
+  <si>
+    <t>Q1 January-March</t>
+  </si>
+  <si>
+    <t>Q2 April-June</t>
+  </si>
+  <si>
+    <t>Q3 July-September</t>
+  </si>
+  <si>
+    <t>Q4 October-December</t>
+  </si>
+  <si>
+    <t>Accomplished</t>
+  </si>
+  <si>
+    <t>CCS Research- Santa Cruz</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>Target Presentation</t>
+  </si>
+  <si>
+    <t>Accomplishment Presentation</t>
+  </si>
+  <si>
+    <t>Target Research Publication</t>
+  </si>
+  <si>
+    <t>Accomplishment Research Publication</t>
+  </si>
+  <si>
+    <t>Target of Research Output Utilized</t>
+  </si>
+  <si>
+    <t>Accomplishment of Research Output Utilized</t>
+  </si>
+  <si>
+    <t>RESEARCH</t>
+  </si>
+  <si>
+    <t>Research Proposal submitted/activity conducted</t>
+  </si>
+  <si>
+    <t>Research Implemented and/or Completed within the timeframe</t>
+  </si>
+  <si>
+    <t>Research Presented in Regional/national/International</t>
+  </si>
+  <si>
+    <t>Filed/Publsihed/Approved IP Rights</t>
+  </si>
+  <si>
+    <t>Research Utilized/Deployed through commercialization/extension policy</t>
+  </si>
+  <si>
+    <t>Number of citations in journals/book</t>
+  </si>
+  <si>
+    <t>Faculty</t>
+  </si>
+  <si>
+    <t>Citations</t>
+  </si>
+  <si>
+    <t>Scopus</t>
+  </si>
+  <si>
+    <t>RG</t>
+  </si>
+  <si>
+    <t>GS</t>
+  </si>
+  <si>
+    <t>2025 CCS Accomplishment Report</t>
+  </si>
+  <si>
+    <t>1st Qtr (January - March)</t>
+  </si>
+  <si>
+    <t>2nd Qtr (April - June)</t>
+  </si>
+  <si>
+    <t>3rd Qtr (July-September)</t>
+  </si>
+  <si>
+    <t>4th Qtr (October-December)</t>
+  </si>
+  <si>
+    <t>SEMESTER/ ACADEMIC YEAR</t>
+  </si>
+  <si>
+    <t>Title of Projects</t>
+  </si>
+  <si>
+    <t>Date / Duration</t>
+  </si>
+  <si>
+    <t>Beneficiaries</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>Extensionists</t>
+  </si>
+  <si>
+    <t>Budget Allocation</t>
+  </si>
+  <si>
+    <t>Evaluation</t>
+  </si>
+  <si>
+    <t>Reference</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">COLLEGE OF COMPUTER STUDIES
+Santa Cruz Campus
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="13"/>
+        <color rgb="FF783F04"/>
+        <rFont val="Poppins"/>
+      </rPr>
+      <t>JANUARY TO MARCH 2025</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="Poppins"/>
+      </rPr>
+      <t xml:space="preserve">
+ FACULTY SEMINAR, CONFERENCE AND TRAINING
+</t>
+    </r>
+  </si>
+  <si>
+    <t>Q1</t>
+  </si>
 </sst>
 </file>
 
@@ -192,7 +396,7 @@
     <numFmt numFmtId="165" formatCode="mmmm\ d\,\ yyyy"/>
     <numFmt numFmtId="166" formatCode="mmmm\ dd\,\ yyyy"/>
   </numFmts>
-  <fonts count="28" x14ac:knownFonts="1">
+  <fonts count="41" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -354,8 +558,85 @@
       <color rgb="FF783F04"/>
       <name val="Poppins"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Poppins"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Poppins"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Poppins"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Poppins"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Poppins"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FF000000"/>
+      <name val="Poppins"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Poppins"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Poppins"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Poppins"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF434343"/>
+      <name val="Poppins"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF434343"/>
+      <name val="Poppins"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="19">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -392,8 +673,80 @@
         <bgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEAD1DC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC9DAF8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB4A7D6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF4CCCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCFE2F3"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEFEFEF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD5A6BD"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6E0B4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF5B3F86"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF6F8F9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="27">
     <border>
       <left/>
       <right/>
@@ -442,11 +795,333 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF442F65"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF5B3F86"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF442F65"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF442F65"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF5B3F86"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF442F65"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF442F65"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF442F65"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF442F65"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF442F65"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF442F65"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFF6F8F9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFF6F8F9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF442F65"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFF6F8F9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF442F65"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFF6F8F9"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFF6F8F9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFF6F8F9"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFF6F8F9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFF6F8F9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="161">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -584,12 +1259,343 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="13" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="11" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="15" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="14" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="11" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="14" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="17" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="17" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="17" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="8" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="8" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="39" fillId="8" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="8" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="8" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="8" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="18" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="18" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="39" fillId="18" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="18" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="18" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="18" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="8" borderId="26" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="18" borderId="26" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="18" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="8" borderId="23" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="18" borderId="23" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="8" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="18" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="18" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="14" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="14" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="4">
@@ -868,46 +1874,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="102.75" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="49" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="50"/>
-      <c r="C1" s="50"/>
-      <c r="D1" s="50"/>
-      <c r="E1" s="50"/>
-      <c r="F1" s="50"/>
-      <c r="G1" s="50"/>
-      <c r="H1" s="50"/>
+      <c r="A1" s="153" t="s">
+        <v>80</v>
+      </c>
+      <c r="B1" s="154"/>
+      <c r="C1" s="154"/>
+      <c r="D1" s="154"/>
+      <c r="E1" s="154"/>
+      <c r="F1" s="154"/>
+      <c r="G1" s="154"/>
+      <c r="H1" s="154"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
     </row>
     <row r="2" spans="1:10" ht="108.75" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="I2" s="5" t="s">
         <v>8</v>
-      </c>
-      <c r="I2" s="5" t="s">
-        <v>9</v>
       </c>
       <c r="J2" s="1"/>
     </row>
@@ -1424,46 +2430,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="102.75" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="49" t="s">
-        <v>10</v>
-      </c>
-      <c r="B1" s="50"/>
-      <c r="C1" s="50"/>
-      <c r="D1" s="50"/>
-      <c r="E1" s="50"/>
-      <c r="F1" s="50"/>
-      <c r="G1" s="50"/>
-      <c r="H1" s="50"/>
+      <c r="A1" s="153" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="154"/>
+      <c r="C1" s="154"/>
+      <c r="D1" s="154"/>
+      <c r="E1" s="154"/>
+      <c r="F1" s="154"/>
+      <c r="G1" s="154"/>
+      <c r="H1" s="154"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
     </row>
     <row r="2" spans="1:10" ht="108.75" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="I2" s="5" t="s">
         <v>8</v>
-      </c>
-      <c r="I2" s="5" t="s">
-        <v>9</v>
       </c>
       <c r="J2" s="1"/>
     </row>
@@ -1984,46 +2990,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="102.75" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="49" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="50"/>
-      <c r="C1" s="50"/>
-      <c r="D1" s="50"/>
-      <c r="E1" s="50"/>
-      <c r="F1" s="50"/>
-      <c r="G1" s="50"/>
-      <c r="H1" s="50"/>
+      <c r="A1" s="153" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="154"/>
+      <c r="C1" s="154"/>
+      <c r="D1" s="154"/>
+      <c r="E1" s="154"/>
+      <c r="F1" s="154"/>
+      <c r="G1" s="154"/>
+      <c r="H1" s="154"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
     </row>
     <row r="2" spans="1:10" ht="108.75" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="I2" s="5" t="s">
         <v>8</v>
-      </c>
-      <c r="I2" s="5" t="s">
-        <v>9</v>
       </c>
       <c r="J2" s="1"/>
     </row>
@@ -2544,46 +3550,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="102.75" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="49" t="s">
-        <v>12</v>
-      </c>
-      <c r="B1" s="50"/>
-      <c r="C1" s="50"/>
-      <c r="D1" s="50"/>
-      <c r="E1" s="50"/>
-      <c r="F1" s="50"/>
-      <c r="G1" s="50"/>
-      <c r="H1" s="50"/>
+      <c r="A1" s="153" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="154"/>
+      <c r="C1" s="154"/>
+      <c r="D1" s="154"/>
+      <c r="E1" s="154"/>
+      <c r="F1" s="154"/>
+      <c r="G1" s="154"/>
+      <c r="H1" s="154"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
     </row>
     <row r="2" spans="1:10" ht="108.75" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="I2" s="5" t="s">
         <v>8</v>
-      </c>
-      <c r="I2" s="5" t="s">
-        <v>9</v>
       </c>
       <c r="J2" s="1"/>
     </row>
@@ -3086,4 +4092,1796 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C961861-FF09-4FB2-A9A3-30B48BF3DE29}">
+  <dimension ref="A1:AD24"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="48.42578125" customWidth="1"/>
+    <col min="2" max="2" width="32.42578125" customWidth="1"/>
+    <col min="3" max="3" width="36.5703125" customWidth="1"/>
+    <col min="4" max="4" width="32.5703125" customWidth="1"/>
+    <col min="5" max="5" width="28.5703125" customWidth="1"/>
+    <col min="6" max="6" width="25.28515625" customWidth="1"/>
+    <col min="7" max="7" width="27.140625" customWidth="1"/>
+    <col min="8" max="8" width="21.5703125" customWidth="1"/>
+    <col min="9" max="9" width="24.85546875" customWidth="1"/>
+    <col min="10" max="10" width="22.42578125" customWidth="1"/>
+    <col min="18" max="18" width="34" customWidth="1"/>
+    <col min="19" max="19" width="37" customWidth="1"/>
+    <col min="20" max="20" width="24.7109375" customWidth="1"/>
+    <col min="21" max="21" width="23.42578125" customWidth="1"/>
+    <col min="22" max="22" width="24.140625" customWidth="1"/>
+    <col min="25" max="25" width="24.42578125" customWidth="1"/>
+    <col min="26" max="26" width="25.140625" customWidth="1"/>
+    <col min="27" max="27" width="14.42578125" customWidth="1"/>
+    <col min="28" max="28" width="26.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:30" ht="29.25" thickBot="1" x14ac:dyDescent="0.85">
+      <c r="A1" s="146" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="147"/>
+      <c r="C1" s="147"/>
+      <c r="D1" s="147"/>
+      <c r="E1" s="147"/>
+      <c r="F1" s="147"/>
+      <c r="G1" s="147"/>
+      <c r="H1" s="147"/>
+      <c r="I1" s="147"/>
+      <c r="J1" s="147"/>
+      <c r="K1" s="147"/>
+      <c r="L1" s="148"/>
+      <c r="M1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:30" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.65">
+      <c r="A2" s="88" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" s="89"/>
+      <c r="C2" s="158" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2" s="159"/>
+      <c r="E2" s="160"/>
+      <c r="F2" s="90"/>
+      <c r="G2" s="49"/>
+      <c r="H2" s="49"/>
+      <c r="I2" s="49"/>
+      <c r="J2" s="49"/>
+      <c r="K2" s="49"/>
+      <c r="L2" s="49"/>
+    </row>
+    <row r="3" spans="1:30" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.65">
+      <c r="A3" s="88" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" s="91"/>
+      <c r="C3" s="158" t="s">
+        <v>51</v>
+      </c>
+      <c r="D3" s="159"/>
+      <c r="E3" s="160"/>
+      <c r="F3" s="89"/>
+      <c r="G3" s="49"/>
+      <c r="H3" s="49"/>
+      <c r="I3" s="49"/>
+      <c r="J3" s="49"/>
+      <c r="K3" s="49"/>
+      <c r="L3" s="49"/>
+    </row>
+    <row r="4" spans="1:30" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.65">
+      <c r="A4" s="88" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" s="91"/>
+      <c r="C4" s="158" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4" s="159"/>
+      <c r="E4" s="160"/>
+      <c r="F4" s="89"/>
+      <c r="G4" s="49"/>
+      <c r="H4" s="49"/>
+      <c r="I4" s="49"/>
+      <c r="J4" s="49"/>
+      <c r="K4" s="49"/>
+      <c r="L4" s="49"/>
+    </row>
+    <row r="5" spans="1:30" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="92"/>
+      <c r="B5" s="92"/>
+      <c r="C5" s="92"/>
+      <c r="D5" s="92"/>
+      <c r="E5" s="58"/>
+      <c r="F5" s="58"/>
+      <c r="G5" s="92"/>
+      <c r="H5" s="92"/>
+      <c r="I5" s="92"/>
+      <c r="J5" s="92"/>
+      <c r="K5" s="49"/>
+      <c r="L5" s="49"/>
+    </row>
+    <row r="6" spans="1:30" ht="41.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="93" t="s">
+        <v>54</v>
+      </c>
+      <c r="B6" s="94"/>
+      <c r="C6" s="94"/>
+      <c r="D6" s="94"/>
+      <c r="E6" s="94"/>
+      <c r="F6" s="94"/>
+      <c r="G6" s="94"/>
+      <c r="H6" s="94"/>
+      <c r="I6" s="94"/>
+      <c r="J6" s="94"/>
+      <c r="K6" s="49"/>
+      <c r="L6" s="49"/>
+      <c r="U6" s="154"/>
+      <c r="V6" s="154"/>
+    </row>
+    <row r="7" spans="1:30" ht="67.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="95" t="s">
+        <v>55</v>
+      </c>
+      <c r="B7" s="125"/>
+      <c r="C7" s="125"/>
+      <c r="D7" s="125"/>
+      <c r="E7" s="125"/>
+      <c r="F7" s="125"/>
+      <c r="G7" s="125"/>
+      <c r="H7" s="125"/>
+      <c r="I7" s="125"/>
+      <c r="J7" s="125"/>
+      <c r="K7" s="49"/>
+      <c r="L7" s="49"/>
+      <c r="U7" s="154"/>
+      <c r="V7" s="154"/>
+    </row>
+    <row r="8" spans="1:30" ht="49.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
+      <c r="A8" s="95" t="s">
+        <v>56</v>
+      </c>
+      <c r="B8" s="125"/>
+      <c r="C8" s="126"/>
+      <c r="D8" s="125"/>
+      <c r="E8" s="125"/>
+      <c r="F8" s="126"/>
+      <c r="G8" s="125"/>
+      <c r="H8" s="126"/>
+      <c r="I8" s="125"/>
+      <c r="J8" s="125"/>
+      <c r="K8" s="96"/>
+      <c r="L8" s="49"/>
+    </row>
+    <row r="9" spans="1:30" ht="41.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
+      <c r="A9" s="95" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" s="125"/>
+      <c r="C9" s="125"/>
+      <c r="D9" s="126"/>
+      <c r="E9" s="125"/>
+      <c r="F9" s="125"/>
+      <c r="G9" s="125"/>
+      <c r="H9" s="125"/>
+      <c r="I9" s="125"/>
+      <c r="J9" s="125"/>
+      <c r="K9" s="96"/>
+      <c r="L9" s="49"/>
+    </row>
+    <row r="10" spans="1:30" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
+      <c r="A10" s="95" t="s">
+        <v>58</v>
+      </c>
+      <c r="B10" s="126"/>
+      <c r="C10" s="125"/>
+      <c r="D10" s="126"/>
+      <c r="E10" s="126"/>
+      <c r="F10" s="125"/>
+      <c r="G10" s="125"/>
+      <c r="H10" s="125"/>
+      <c r="I10" s="125"/>
+      <c r="J10" s="126"/>
+      <c r="K10" s="96"/>
+      <c r="L10" s="49"/>
+    </row>
+    <row r="11" spans="1:30" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
+      <c r="A11" s="95" t="s">
+        <v>59</v>
+      </c>
+      <c r="B11" s="125"/>
+      <c r="C11" s="125"/>
+      <c r="D11" s="125"/>
+      <c r="E11" s="125"/>
+      <c r="F11" s="125"/>
+      <c r="G11" s="125"/>
+      <c r="H11" s="125"/>
+      <c r="I11" s="125"/>
+      <c r="J11" s="125"/>
+      <c r="K11" s="96"/>
+      <c r="L11" s="49"/>
+    </row>
+    <row r="12" spans="1:30" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
+      <c r="A12" s="95" t="s">
+        <v>60</v>
+      </c>
+      <c r="B12" s="125"/>
+      <c r="C12" s="125"/>
+      <c r="D12" s="125"/>
+      <c r="E12" s="125"/>
+      <c r="F12" s="125"/>
+      <c r="G12" s="125"/>
+      <c r="H12" s="125"/>
+      <c r="I12" s="125"/>
+      <c r="J12" s="125"/>
+      <c r="K12" s="96"/>
+      <c r="L12" s="49"/>
+    </row>
+    <row r="13" spans="1:30" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="49"/>
+      <c r="B13" s="49"/>
+      <c r="C13" s="49"/>
+      <c r="D13" s="49"/>
+      <c r="E13" s="49"/>
+      <c r="F13" s="49"/>
+      <c r="G13" s="49"/>
+      <c r="H13" s="49"/>
+      <c r="I13" s="49"/>
+      <c r="J13" s="49"/>
+      <c r="K13" s="49"/>
+      <c r="L13" s="49"/>
+      <c r="Z13" s="49"/>
+      <c r="AA13" s="49"/>
+      <c r="AB13" s="49"/>
+      <c r="AC13" s="49"/>
+      <c r="AD13" s="49"/>
+    </row>
+    <row r="14" spans="1:30" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="52"/>
+      <c r="B14" s="52"/>
+      <c r="C14" s="52"/>
+      <c r="D14" s="52"/>
+      <c r="E14" s="49"/>
+      <c r="F14" s="49"/>
+      <c r="G14" s="49"/>
+      <c r="H14" s="49"/>
+      <c r="I14" s="49"/>
+      <c r="J14" s="49"/>
+      <c r="K14" s="49"/>
+      <c r="L14" s="49"/>
+      <c r="Z14" s="49"/>
+      <c r="AA14" s="49"/>
+      <c r="AB14" s="49"/>
+      <c r="AC14" s="49"/>
+      <c r="AD14" s="49"/>
+    </row>
+    <row r="15" spans="1:30" ht="24" thickBot="1" x14ac:dyDescent="0.65">
+      <c r="A15" s="88" t="s">
+        <v>61</v>
+      </c>
+      <c r="B15" s="155" t="s">
+        <v>62</v>
+      </c>
+      <c r="C15" s="156"/>
+      <c r="D15" s="157"/>
+      <c r="E15" s="49"/>
+      <c r="F15" s="49"/>
+      <c r="G15" s="49"/>
+      <c r="H15" s="49"/>
+      <c r="I15" s="49"/>
+      <c r="J15" s="49"/>
+      <c r="K15" s="49"/>
+      <c r="L15" s="49"/>
+      <c r="Z15" s="49"/>
+      <c r="AA15" s="49"/>
+      <c r="AB15" s="49"/>
+      <c r="AC15" s="49"/>
+      <c r="AD15" s="49"/>
+    </row>
+    <row r="16" spans="1:30" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="97"/>
+      <c r="B16" s="98" t="s">
+        <v>63</v>
+      </c>
+      <c r="C16" s="98" t="s">
+        <v>64</v>
+      </c>
+      <c r="D16" s="98" t="s">
+        <v>65</v>
+      </c>
+      <c r="E16" s="49"/>
+      <c r="F16" s="49"/>
+      <c r="G16" s="49"/>
+      <c r="H16" s="49"/>
+      <c r="I16" s="49"/>
+      <c r="J16" s="49"/>
+      <c r="K16" s="49"/>
+      <c r="L16" s="49"/>
+      <c r="Z16" s="49"/>
+      <c r="AA16" s="49"/>
+      <c r="AB16" s="49"/>
+      <c r="AC16" s="49"/>
+      <c r="AD16" s="49"/>
+    </row>
+    <row r="17" spans="1:30" ht="24" thickBot="1" x14ac:dyDescent="0.7">
+      <c r="A17" s="97"/>
+      <c r="B17" s="99"/>
+      <c r="C17" s="99"/>
+      <c r="D17" s="99"/>
+      <c r="E17" s="49"/>
+      <c r="F17" s="49"/>
+      <c r="G17" s="49"/>
+      <c r="H17" s="49"/>
+      <c r="I17" s="49"/>
+      <c r="J17" s="49"/>
+      <c r="K17" s="49"/>
+      <c r="L17" s="49"/>
+      <c r="Z17" s="49"/>
+      <c r="AA17" s="49"/>
+      <c r="AB17" s="49"/>
+      <c r="AC17" s="49"/>
+      <c r="AD17" s="49"/>
+    </row>
+    <row r="18" spans="1:30" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="49"/>
+      <c r="B18" s="49"/>
+      <c r="C18" s="49"/>
+      <c r="D18" s="49"/>
+      <c r="E18" s="49"/>
+      <c r="F18" s="49"/>
+      <c r="G18" s="49"/>
+      <c r="H18" s="49"/>
+      <c r="I18" s="49"/>
+      <c r="J18" s="49"/>
+      <c r="K18" s="49"/>
+      <c r="L18" s="49"/>
+      <c r="Z18" s="49"/>
+      <c r="AA18" s="49"/>
+      <c r="AB18" s="49"/>
+      <c r="AC18" s="49"/>
+      <c r="AD18" s="49"/>
+    </row>
+    <row r="19" spans="1:30" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="49"/>
+      <c r="B19" s="49"/>
+      <c r="C19" s="49"/>
+      <c r="D19" s="49"/>
+      <c r="E19" s="49"/>
+      <c r="F19" s="49"/>
+      <c r="G19" s="49"/>
+      <c r="H19" s="49"/>
+      <c r="I19" s="49"/>
+      <c r="J19" s="49"/>
+      <c r="K19" s="49"/>
+      <c r="L19" s="49"/>
+      <c r="Z19" s="49"/>
+      <c r="AA19" s="49"/>
+      <c r="AB19" s="49"/>
+      <c r="AC19" s="49"/>
+      <c r="AD19" s="49"/>
+    </row>
+    <row r="20" spans="1:30" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A20" s="100" t="s">
+        <v>66</v>
+      </c>
+      <c r="B20" s="49"/>
+      <c r="C20" s="49"/>
+      <c r="D20" s="49"/>
+      <c r="E20" s="49"/>
+      <c r="F20" s="49"/>
+      <c r="G20" s="49"/>
+      <c r="H20" s="49"/>
+      <c r="I20" s="49"/>
+      <c r="J20" s="49"/>
+      <c r="K20" s="49"/>
+      <c r="L20" s="49"/>
+      <c r="Z20" s="49"/>
+      <c r="AA20" s="49"/>
+      <c r="AB20" s="49"/>
+      <c r="AC20" s="49"/>
+      <c r="AD20" s="49"/>
+    </row>
+    <row r="21" spans="1:30" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A21" s="67" t="s">
+        <v>67</v>
+      </c>
+      <c r="B21" s="101"/>
+      <c r="C21" s="49"/>
+      <c r="D21" s="49"/>
+      <c r="E21" s="49"/>
+      <c r="F21" s="49"/>
+      <c r="G21" s="49"/>
+      <c r="H21" s="49"/>
+      <c r="I21" s="49"/>
+      <c r="J21" s="49"/>
+      <c r="K21" s="49"/>
+      <c r="L21" s="49"/>
+      <c r="Z21" s="49"/>
+      <c r="AA21" s="49"/>
+      <c r="AB21" s="49"/>
+      <c r="AC21" s="49"/>
+      <c r="AD21" s="49"/>
+    </row>
+    <row r="22" spans="1:30" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A22" s="67" t="s">
+        <v>68</v>
+      </c>
+      <c r="B22" s="101"/>
+      <c r="C22" s="49"/>
+      <c r="D22" s="49"/>
+      <c r="E22" s="49"/>
+      <c r="F22" s="49"/>
+      <c r="G22" s="49"/>
+      <c r="H22" s="49"/>
+      <c r="I22" s="49"/>
+      <c r="J22" s="49"/>
+      <c r="K22" s="49"/>
+      <c r="L22" s="49"/>
+      <c r="Z22" s="49"/>
+      <c r="AA22" s="49"/>
+      <c r="AB22" s="49"/>
+      <c r="AC22" s="49"/>
+      <c r="AD22" s="49"/>
+    </row>
+    <row r="23" spans="1:30" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A23" s="67" t="s">
+        <v>69</v>
+      </c>
+      <c r="B23" s="101"/>
+      <c r="C23" s="49"/>
+      <c r="D23" s="49"/>
+      <c r="E23" s="49"/>
+      <c r="F23" s="49"/>
+      <c r="G23" s="49"/>
+      <c r="H23" s="49"/>
+      <c r="I23" s="49"/>
+      <c r="J23" s="49"/>
+      <c r="K23" s="49"/>
+      <c r="L23" s="49"/>
+      <c r="Z23" s="49"/>
+      <c r="AA23" s="49"/>
+      <c r="AB23" s="49"/>
+      <c r="AC23" s="49"/>
+      <c r="AD23" s="49"/>
+    </row>
+    <row r="24" spans="1:30" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A24" s="67" t="s">
+        <v>70</v>
+      </c>
+      <c r="B24" s="101"/>
+      <c r="C24" s="49"/>
+      <c r="D24" s="49"/>
+      <c r="E24" s="49"/>
+      <c r="F24" s="49"/>
+      <c r="G24" s="49"/>
+      <c r="H24" s="49"/>
+      <c r="I24" s="49"/>
+      <c r="J24" s="49"/>
+      <c r="K24" s="49"/>
+      <c r="L24" s="49"/>
+      <c r="Z24" s="49"/>
+      <c r="AA24" s="49"/>
+      <c r="AB24" s="49"/>
+      <c r="AC24" s="49"/>
+      <c r="AD24" s="49"/>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="U6:V6"/>
+    <mergeCell ref="U7:V7"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="C2:E2"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="C4:E4"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1040D8A3-60D0-4196-AE89-D06A14E48956}">
+  <dimension ref="A1:R36"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="38.5703125" customWidth="1"/>
+    <col min="2" max="2" width="22.5703125" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="19.140625" customWidth="1"/>
+    <col min="5" max="5" width="12.140625" customWidth="1"/>
+    <col min="6" max="6" width="17" customWidth="1"/>
+    <col min="7" max="7" width="22.140625" customWidth="1"/>
+    <col min="8" max="8" width="17" customWidth="1"/>
+    <col min="9" max="9" width="23.7109375" customWidth="1"/>
+    <col min="10" max="10" width="21" customWidth="1"/>
+    <col min="11" max="11" width="13.140625" customWidth="1"/>
+    <col min="12" max="12" width="18.5703125" customWidth="1"/>
+    <col min="13" max="13" width="14.5703125" customWidth="1"/>
+    <col min="15" max="15" width="14" customWidth="1"/>
+    <col min="18" max="18" width="14.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18" ht="29.25" thickBot="1" x14ac:dyDescent="0.85">
+      <c r="A1" s="146" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="147"/>
+      <c r="C1" s="147"/>
+      <c r="D1" s="147"/>
+      <c r="E1" s="147"/>
+      <c r="F1" s="147"/>
+      <c r="G1" s="147"/>
+      <c r="H1" s="147"/>
+      <c r="I1" s="147"/>
+      <c r="J1" s="147"/>
+      <c r="K1" s="147"/>
+      <c r="L1" s="148"/>
+      <c r="M1" s="49"/>
+      <c r="N1" s="49"/>
+      <c r="O1" s="49"/>
+      <c r="P1" s="49"/>
+      <c r="Q1" s="49"/>
+      <c r="R1" s="49"/>
+    </row>
+    <row r="2" spans="1:18" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.7">
+      <c r="A2" s="149" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="150"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="49"/>
+      <c r="F2" s="49"/>
+      <c r="G2" s="51"/>
+      <c r="H2" s="51"/>
+      <c r="I2" s="49"/>
+      <c r="J2" s="51"/>
+      <c r="K2" s="51"/>
+      <c r="L2" s="49"/>
+      <c r="M2" s="49"/>
+      <c r="N2" s="49"/>
+      <c r="O2" s="49"/>
+      <c r="P2" s="49"/>
+      <c r="Q2" s="49"/>
+      <c r="R2" s="49"/>
+    </row>
+    <row r="3" spans="1:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="52"/>
+      <c r="B3" s="52"/>
+      <c r="C3" s="52"/>
+      <c r="D3" s="49"/>
+      <c r="E3" s="49"/>
+      <c r="F3" s="49"/>
+      <c r="G3" s="51"/>
+      <c r="H3" s="51"/>
+      <c r="I3" s="49"/>
+      <c r="J3" s="51"/>
+      <c r="K3" s="51"/>
+      <c r="L3" s="49"/>
+      <c r="M3" s="49"/>
+      <c r="N3" s="49"/>
+      <c r="O3" s="49"/>
+      <c r="P3" s="49"/>
+      <c r="Q3" s="49"/>
+      <c r="R3" s="49"/>
+    </row>
+    <row r="4" spans="1:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="52"/>
+      <c r="B4" s="52"/>
+      <c r="C4" s="52"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="52"/>
+      <c r="F4" s="52"/>
+      <c r="G4" s="52"/>
+      <c r="H4" s="52"/>
+      <c r="I4" s="52"/>
+      <c r="J4" s="52"/>
+      <c r="K4" s="52"/>
+      <c r="L4" s="52"/>
+      <c r="M4" s="49"/>
+      <c r="N4" s="49"/>
+      <c r="O4" s="49"/>
+      <c r="P4" s="49"/>
+      <c r="Q4" s="49"/>
+      <c r="R4" s="49"/>
+    </row>
+    <row r="5" spans="1:18" ht="39.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="53" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="54" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="151" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="152"/>
+      <c r="E5" s="138" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" s="139"/>
+      <c r="G5" s="142" t="s">
+        <v>18</v>
+      </c>
+      <c r="H5" s="143"/>
+      <c r="I5" s="144" t="s">
+        <v>19</v>
+      </c>
+      <c r="J5" s="145"/>
+      <c r="K5" s="54" t="s">
+        <v>20</v>
+      </c>
+      <c r="L5" s="54" t="s">
+        <v>21</v>
+      </c>
+      <c r="M5" s="55"/>
+      <c r="N5" s="55"/>
+      <c r="O5" s="55"/>
+      <c r="P5" s="55"/>
+      <c r="Q5" s="55"/>
+      <c r="R5" s="55"/>
+    </row>
+    <row r="6" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="56"/>
+      <c r="B6" s="57"/>
+      <c r="C6" s="54" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="54" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" s="54" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" s="54" t="s">
+        <v>23</v>
+      </c>
+      <c r="G6" s="54" t="s">
+        <v>22</v>
+      </c>
+      <c r="H6" s="54" t="s">
+        <v>23</v>
+      </c>
+      <c r="I6" s="54" t="s">
+        <v>22</v>
+      </c>
+      <c r="J6" s="54" t="s">
+        <v>23</v>
+      </c>
+      <c r="K6" s="58"/>
+      <c r="L6" s="58"/>
+      <c r="M6" s="55"/>
+      <c r="N6" s="55"/>
+      <c r="O6" s="55"/>
+      <c r="P6" s="55"/>
+      <c r="Q6" s="55"/>
+      <c r="R6" s="55"/>
+    </row>
+    <row r="7" spans="1:18" ht="50.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A7" s="127" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="59" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="60"/>
+      <c r="D7" s="60"/>
+      <c r="E7" s="60"/>
+      <c r="F7" s="57"/>
+      <c r="G7" s="60"/>
+      <c r="H7" s="57"/>
+      <c r="I7" s="60"/>
+      <c r="J7" s="57"/>
+      <c r="K7" s="60"/>
+      <c r="L7" s="60"/>
+      <c r="M7" s="49"/>
+      <c r="N7" s="49"/>
+      <c r="O7" s="49"/>
+      <c r="P7" s="49"/>
+      <c r="Q7" s="49"/>
+      <c r="R7" s="49"/>
+    </row>
+    <row r="8" spans="1:18" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A8" s="128"/>
+      <c r="B8" s="61" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="60"/>
+      <c r="D8" s="60"/>
+      <c r="E8" s="60"/>
+      <c r="F8" s="57"/>
+      <c r="G8" s="60"/>
+      <c r="H8" s="57"/>
+      <c r="I8" s="60"/>
+      <c r="J8" s="57"/>
+      <c r="K8" s="60"/>
+      <c r="L8" s="60"/>
+      <c r="M8" s="49"/>
+      <c r="N8" s="49"/>
+      <c r="O8" s="49"/>
+      <c r="P8" s="49"/>
+      <c r="Q8" s="49"/>
+      <c r="R8" s="49"/>
+    </row>
+    <row r="9" spans="1:18" ht="39.75" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A9" s="129"/>
+      <c r="B9" s="61" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="60"/>
+      <c r="D9" s="60"/>
+      <c r="E9" s="60"/>
+      <c r="F9" s="57"/>
+      <c r="G9" s="60"/>
+      <c r="H9" s="57"/>
+      <c r="I9" s="60"/>
+      <c r="J9" s="57"/>
+      <c r="K9" s="60"/>
+      <c r="L9" s="60"/>
+      <c r="M9" s="49"/>
+      <c r="N9" s="49"/>
+      <c r="O9" s="49"/>
+      <c r="P9" s="49"/>
+      <c r="Q9" s="49"/>
+      <c r="R9" s="49"/>
+    </row>
+    <row r="10" spans="1:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="49"/>
+      <c r="B10" s="49"/>
+      <c r="C10" s="49"/>
+      <c r="D10" s="49"/>
+      <c r="E10" s="49"/>
+      <c r="F10" s="49"/>
+      <c r="G10" s="49"/>
+      <c r="H10" s="49"/>
+      <c r="I10" s="49"/>
+      <c r="J10" s="49"/>
+      <c r="K10" s="49"/>
+      <c r="L10" s="49"/>
+      <c r="M10" s="49"/>
+      <c r="N10" s="49"/>
+      <c r="O10" s="49"/>
+      <c r="P10" s="49"/>
+      <c r="Q10" s="49"/>
+      <c r="R10" s="49"/>
+    </row>
+    <row r="11" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A11" s="62" t="s">
+        <v>28</v>
+      </c>
+      <c r="B11" s="63"/>
+      <c r="C11" s="49"/>
+      <c r="D11" s="49"/>
+      <c r="E11" s="49"/>
+      <c r="F11" s="49"/>
+      <c r="G11" s="49"/>
+      <c r="H11" s="49"/>
+      <c r="I11" s="49"/>
+      <c r="J11" s="49"/>
+      <c r="K11" s="49"/>
+      <c r="L11" s="49"/>
+      <c r="M11" s="49"/>
+      <c r="N11" s="49"/>
+      <c r="O11" s="49"/>
+      <c r="P11" s="49"/>
+      <c r="Q11" s="49"/>
+      <c r="R11" s="49"/>
+    </row>
+    <row r="12" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="64" t="s">
+        <v>29</v>
+      </c>
+      <c r="B12" s="63"/>
+      <c r="C12" s="49"/>
+      <c r="D12" s="49"/>
+      <c r="E12" s="49"/>
+      <c r="F12" s="49"/>
+      <c r="G12" s="49"/>
+      <c r="H12" s="49"/>
+      <c r="I12" s="49"/>
+      <c r="J12" s="49"/>
+      <c r="K12" s="49"/>
+      <c r="L12" s="49"/>
+      <c r="M12" s="49"/>
+      <c r="N12" s="49"/>
+      <c r="O12" s="49"/>
+      <c r="P12" s="49"/>
+      <c r="Q12" s="49"/>
+      <c r="R12" s="49"/>
+    </row>
+    <row r="13" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="64" t="s">
+        <v>30</v>
+      </c>
+      <c r="B13" s="63"/>
+      <c r="C13" s="49"/>
+      <c r="D13" s="49"/>
+      <c r="E13" s="49"/>
+      <c r="F13" s="49"/>
+      <c r="G13" s="49"/>
+      <c r="H13" s="49"/>
+      <c r="I13" s="49"/>
+      <c r="J13" s="49"/>
+      <c r="K13" s="49"/>
+      <c r="L13" s="49"/>
+      <c r="M13" s="49"/>
+      <c r="N13" s="49"/>
+      <c r="O13" s="49"/>
+      <c r="P13" s="49"/>
+      <c r="Q13" s="49"/>
+      <c r="R13" s="49"/>
+    </row>
+    <row r="14" spans="1:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="49"/>
+      <c r="B14" s="49"/>
+      <c r="C14" s="49"/>
+      <c r="D14" s="49"/>
+      <c r="E14" s="49"/>
+      <c r="F14" s="49"/>
+      <c r="G14" s="49"/>
+      <c r="H14" s="49"/>
+      <c r="I14" s="49"/>
+      <c r="J14" s="49"/>
+      <c r="K14" s="49"/>
+      <c r="L14" s="49"/>
+      <c r="M14" s="49"/>
+      <c r="N14" s="49"/>
+      <c r="O14" s="49"/>
+      <c r="P14" s="49"/>
+      <c r="Q14" s="49"/>
+      <c r="R14" s="49"/>
+    </row>
+    <row r="15" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A15" s="66" t="s">
+        <v>81</v>
+      </c>
+      <c r="B15" s="49"/>
+      <c r="C15" s="66" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15" s="49"/>
+      <c r="E15" s="49"/>
+      <c r="F15" s="66" t="s">
+        <v>32</v>
+      </c>
+      <c r="G15" s="49"/>
+      <c r="H15" s="66" t="s">
+        <v>33</v>
+      </c>
+      <c r="I15" s="49"/>
+      <c r="J15" s="49"/>
+      <c r="K15" s="49"/>
+      <c r="L15" s="49"/>
+      <c r="M15" s="49"/>
+      <c r="N15" s="49"/>
+      <c r="O15" s="49"/>
+      <c r="P15" s="49"/>
+      <c r="Q15" s="49"/>
+      <c r="R15" s="49"/>
+    </row>
+    <row r="16" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A16" s="67"/>
+      <c r="B16" s="49"/>
+      <c r="C16" s="67"/>
+      <c r="D16" s="49"/>
+      <c r="E16" s="49"/>
+      <c r="F16" s="67"/>
+      <c r="G16" s="49"/>
+      <c r="H16" s="65"/>
+      <c r="I16" s="49"/>
+      <c r="J16" s="49"/>
+      <c r="K16" s="49"/>
+      <c r="L16" s="49"/>
+      <c r="M16" s="49"/>
+      <c r="N16" s="49"/>
+      <c r="O16" s="49"/>
+      <c r="P16" s="49"/>
+      <c r="Q16" s="49"/>
+      <c r="R16" s="49"/>
+    </row>
+    <row r="17" spans="1:18" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A17" s="68"/>
+      <c r="B17" s="67" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17" s="68"/>
+      <c r="D17" s="65" t="s">
+        <v>34</v>
+      </c>
+      <c r="E17" s="49"/>
+      <c r="F17" s="68"/>
+      <c r="G17" s="65" t="s">
+        <v>34</v>
+      </c>
+      <c r="H17" s="68"/>
+      <c r="I17" s="65" t="s">
+        <v>34</v>
+      </c>
+      <c r="J17" s="49"/>
+      <c r="K17" s="49"/>
+      <c r="L17" s="49"/>
+      <c r="M17" s="49"/>
+      <c r="N17" s="49"/>
+      <c r="O17" s="49"/>
+      <c r="P17" s="49"/>
+      <c r="Q17" s="49"/>
+      <c r="R17" s="49"/>
+    </row>
+    <row r="18" spans="1:18" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A18" s="68"/>
+      <c r="B18" s="67" t="s">
+        <v>35</v>
+      </c>
+      <c r="C18" s="68"/>
+      <c r="D18" s="65" t="s">
+        <v>35</v>
+      </c>
+      <c r="E18" s="49"/>
+      <c r="F18" s="68"/>
+      <c r="G18" s="65" t="s">
+        <v>35</v>
+      </c>
+      <c r="H18" s="68"/>
+      <c r="I18" s="65" t="s">
+        <v>35</v>
+      </c>
+      <c r="J18" s="49"/>
+      <c r="K18" s="49"/>
+      <c r="L18" s="49"/>
+      <c r="M18" s="49"/>
+      <c r="N18" s="49"/>
+      <c r="O18" s="49"/>
+      <c r="P18" s="49"/>
+      <c r="Q18" s="49"/>
+      <c r="R18" s="49"/>
+    </row>
+    <row r="19" spans="1:18" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A19" s="68"/>
+      <c r="B19" s="67" t="s">
+        <v>36</v>
+      </c>
+      <c r="C19" s="68"/>
+      <c r="D19" s="65" t="s">
+        <v>36</v>
+      </c>
+      <c r="E19" s="49"/>
+      <c r="F19" s="68"/>
+      <c r="G19" s="65" t="s">
+        <v>36</v>
+      </c>
+      <c r="H19" s="68"/>
+      <c r="I19" s="65" t="s">
+        <v>36</v>
+      </c>
+      <c r="J19" s="49"/>
+      <c r="K19" s="49"/>
+      <c r="L19" s="49"/>
+      <c r="M19" s="49"/>
+      <c r="N19" s="49"/>
+      <c r="O19" s="49"/>
+      <c r="P19" s="49"/>
+      <c r="Q19" s="49"/>
+      <c r="R19" s="49"/>
+    </row>
+    <row r="20" spans="1:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="49"/>
+      <c r="B20" s="49"/>
+      <c r="C20" s="49"/>
+      <c r="D20" s="49"/>
+      <c r="E20" s="49"/>
+      <c r="F20" s="49"/>
+      <c r="G20" s="49"/>
+      <c r="H20" s="49"/>
+      <c r="I20" s="49"/>
+      <c r="J20" s="49"/>
+      <c r="K20" s="49"/>
+      <c r="L20" s="49"/>
+      <c r="M20" s="49"/>
+      <c r="N20" s="49"/>
+      <c r="O20" s="49"/>
+      <c r="P20" s="49"/>
+      <c r="Q20" s="49"/>
+      <c r="R20" s="49"/>
+    </row>
+    <row r="21" spans="1:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="52"/>
+      <c r="B21" s="52"/>
+      <c r="C21" s="52"/>
+      <c r="D21" s="52"/>
+      <c r="E21" s="52"/>
+      <c r="F21" s="52"/>
+      <c r="G21" s="52"/>
+      <c r="H21" s="52"/>
+      <c r="I21" s="52"/>
+      <c r="J21" s="52"/>
+      <c r="K21" s="52"/>
+      <c r="L21" s="52"/>
+      <c r="M21" s="52"/>
+      <c r="N21" s="52"/>
+      <c r="O21" s="52"/>
+      <c r="P21" s="52"/>
+      <c r="Q21" s="52"/>
+      <c r="R21" s="52"/>
+    </row>
+    <row r="22" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A22" s="130" t="s">
+        <v>37</v>
+      </c>
+      <c r="B22" s="130" t="s">
+        <v>38</v>
+      </c>
+      <c r="C22" s="133" t="s">
+        <v>39</v>
+      </c>
+      <c r="D22" s="134"/>
+      <c r="E22" s="134"/>
+      <c r="F22" s="134"/>
+      <c r="G22" s="134"/>
+      <c r="H22" s="135"/>
+      <c r="I22" s="57"/>
+      <c r="J22" s="133" t="s">
+        <v>40</v>
+      </c>
+      <c r="K22" s="134"/>
+      <c r="L22" s="134"/>
+      <c r="M22" s="134"/>
+      <c r="N22" s="134"/>
+      <c r="O22" s="135"/>
+      <c r="P22" s="57"/>
+      <c r="Q22" s="133">
+        <v>2025</v>
+      </c>
+      <c r="R22" s="135"/>
+    </row>
+    <row r="23" spans="1:18" ht="39.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="131"/>
+      <c r="B23" s="131"/>
+      <c r="C23" s="136" t="s">
+        <v>41</v>
+      </c>
+      <c r="D23" s="137"/>
+      <c r="E23" s="138" t="s">
+        <v>42</v>
+      </c>
+      <c r="F23" s="139"/>
+      <c r="G23" s="140" t="s">
+        <v>39</v>
+      </c>
+      <c r="H23" s="141"/>
+      <c r="I23" s="58"/>
+      <c r="J23" s="142" t="s">
+        <v>43</v>
+      </c>
+      <c r="K23" s="143"/>
+      <c r="L23" s="144" t="s">
+        <v>44</v>
+      </c>
+      <c r="M23" s="145"/>
+      <c r="N23" s="140" t="s">
+        <v>40</v>
+      </c>
+      <c r="O23" s="141"/>
+      <c r="P23" s="58"/>
+      <c r="Q23" s="69" t="s">
+        <v>20</v>
+      </c>
+      <c r="R23" s="69" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="132"/>
+      <c r="B24" s="132"/>
+      <c r="C24" s="70" t="s">
+        <v>22</v>
+      </c>
+      <c r="D24" s="71" t="s">
+        <v>45</v>
+      </c>
+      <c r="E24" s="70" t="s">
+        <v>22</v>
+      </c>
+      <c r="F24" s="72" t="s">
+        <v>45</v>
+      </c>
+      <c r="G24" s="73" t="s">
+        <v>22</v>
+      </c>
+      <c r="H24" s="73" t="s">
+        <v>45</v>
+      </c>
+      <c r="I24" s="58"/>
+      <c r="J24" s="70" t="s">
+        <v>22</v>
+      </c>
+      <c r="K24" s="74" t="s">
+        <v>45</v>
+      </c>
+      <c r="L24" s="70" t="s">
+        <v>22</v>
+      </c>
+      <c r="M24" s="75" t="s">
+        <v>45</v>
+      </c>
+      <c r="N24" s="73" t="s">
+        <v>22</v>
+      </c>
+      <c r="O24" s="73" t="s">
+        <v>45</v>
+      </c>
+      <c r="P24" s="58"/>
+      <c r="Q24" s="76"/>
+      <c r="R24" s="76"/>
+    </row>
+    <row r="25" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A25" s="77"/>
+      <c r="B25" s="78"/>
+      <c r="C25" s="79"/>
+      <c r="D25" s="80"/>
+      <c r="E25" s="79"/>
+      <c r="F25" s="81"/>
+      <c r="G25" s="82"/>
+      <c r="H25" s="82"/>
+      <c r="I25" s="57"/>
+      <c r="J25" s="79"/>
+      <c r="K25" s="83"/>
+      <c r="L25" s="79"/>
+      <c r="M25" s="84"/>
+      <c r="N25" s="82"/>
+      <c r="O25" s="82"/>
+      <c r="P25" s="57"/>
+      <c r="Q25" s="82"/>
+      <c r="R25" s="82"/>
+    </row>
+    <row r="26" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A26" s="77"/>
+      <c r="B26" s="78"/>
+      <c r="C26" s="79"/>
+      <c r="D26" s="80"/>
+      <c r="E26" s="79"/>
+      <c r="F26" s="81"/>
+      <c r="G26" s="82"/>
+      <c r="H26" s="82"/>
+      <c r="I26" s="57"/>
+      <c r="J26" s="79"/>
+      <c r="K26" s="83"/>
+      <c r="L26" s="79"/>
+      <c r="M26" s="84"/>
+      <c r="N26" s="82"/>
+      <c r="O26" s="82"/>
+      <c r="P26" s="57"/>
+      <c r="Q26" s="82"/>
+      <c r="R26" s="82"/>
+    </row>
+    <row r="27" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A27" s="77"/>
+      <c r="B27" s="78"/>
+      <c r="C27" s="79"/>
+      <c r="D27" s="80"/>
+      <c r="E27" s="79"/>
+      <c r="F27" s="81"/>
+      <c r="G27" s="82"/>
+      <c r="H27" s="82"/>
+      <c r="I27" s="57"/>
+      <c r="J27" s="79"/>
+      <c r="K27" s="83"/>
+      <c r="L27" s="79"/>
+      <c r="M27" s="84"/>
+      <c r="N27" s="82"/>
+      <c r="O27" s="82"/>
+      <c r="P27" s="57"/>
+      <c r="Q27" s="82"/>
+      <c r="R27" s="82"/>
+    </row>
+    <row r="28" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A28" s="77"/>
+      <c r="B28" s="78"/>
+      <c r="C28" s="79"/>
+      <c r="D28" s="80"/>
+      <c r="E28" s="79"/>
+      <c r="F28" s="81"/>
+      <c r="G28" s="82"/>
+      <c r="H28" s="82"/>
+      <c r="I28" s="57"/>
+      <c r="J28" s="79"/>
+      <c r="K28" s="83"/>
+      <c r="L28" s="79"/>
+      <c r="M28" s="84"/>
+      <c r="N28" s="82"/>
+      <c r="O28" s="82"/>
+      <c r="P28" s="57"/>
+      <c r="Q28" s="82"/>
+      <c r="R28" s="82"/>
+    </row>
+    <row r="29" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A29" s="77"/>
+      <c r="B29" s="78"/>
+      <c r="C29" s="79"/>
+      <c r="D29" s="80"/>
+      <c r="E29" s="79"/>
+      <c r="F29" s="81"/>
+      <c r="G29" s="82"/>
+      <c r="H29" s="82"/>
+      <c r="I29" s="57"/>
+      <c r="J29" s="79"/>
+      <c r="K29" s="83"/>
+      <c r="L29" s="79"/>
+      <c r="M29" s="84"/>
+      <c r="N29" s="82"/>
+      <c r="O29" s="82"/>
+      <c r="P29" s="57"/>
+      <c r="Q29" s="82"/>
+      <c r="R29" s="82"/>
+    </row>
+    <row r="30" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A30" s="77"/>
+      <c r="B30" s="78"/>
+      <c r="C30" s="79"/>
+      <c r="D30" s="80"/>
+      <c r="E30" s="79"/>
+      <c r="F30" s="81"/>
+      <c r="G30" s="82"/>
+      <c r="H30" s="82"/>
+      <c r="I30" s="57"/>
+      <c r="J30" s="79"/>
+      <c r="K30" s="83"/>
+      <c r="L30" s="79"/>
+      <c r="M30" s="84"/>
+      <c r="N30" s="82"/>
+      <c r="O30" s="82"/>
+      <c r="P30" s="57"/>
+      <c r="Q30" s="82"/>
+      <c r="R30" s="82"/>
+    </row>
+    <row r="31" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A31" s="77"/>
+      <c r="B31" s="78"/>
+      <c r="C31" s="79"/>
+      <c r="D31" s="80"/>
+      <c r="E31" s="79"/>
+      <c r="F31" s="81"/>
+      <c r="G31" s="82"/>
+      <c r="H31" s="82"/>
+      <c r="I31" s="57"/>
+      <c r="J31" s="79"/>
+      <c r="K31" s="83"/>
+      <c r="L31" s="79"/>
+      <c r="M31" s="84"/>
+      <c r="N31" s="82"/>
+      <c r="O31" s="82"/>
+      <c r="P31" s="57"/>
+      <c r="Q31" s="82"/>
+      <c r="R31" s="82"/>
+    </row>
+    <row r="32" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A32" s="77"/>
+      <c r="B32" s="78"/>
+      <c r="C32" s="79"/>
+      <c r="D32" s="80"/>
+      <c r="E32" s="79"/>
+      <c r="F32" s="81"/>
+      <c r="G32" s="82"/>
+      <c r="H32" s="82"/>
+      <c r="I32" s="57"/>
+      <c r="J32" s="79"/>
+      <c r="K32" s="83"/>
+      <c r="L32" s="79"/>
+      <c r="M32" s="84"/>
+      <c r="N32" s="82"/>
+      <c r="O32" s="82"/>
+      <c r="P32" s="57"/>
+      <c r="Q32" s="82"/>
+      <c r="R32" s="82"/>
+    </row>
+    <row r="33" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A33" s="77"/>
+      <c r="B33" s="78"/>
+      <c r="C33" s="79"/>
+      <c r="D33" s="80"/>
+      <c r="E33" s="79"/>
+      <c r="F33" s="81"/>
+      <c r="G33" s="82"/>
+      <c r="H33" s="82"/>
+      <c r="I33" s="57"/>
+      <c r="J33" s="79"/>
+      <c r="K33" s="83"/>
+      <c r="L33" s="79"/>
+      <c r="M33" s="84"/>
+      <c r="N33" s="82"/>
+      <c r="O33" s="82"/>
+      <c r="P33" s="57"/>
+      <c r="Q33" s="82"/>
+      <c r="R33" s="82"/>
+    </row>
+    <row r="34" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A34" s="49"/>
+      <c r="B34" s="85"/>
+      <c r="C34" s="86"/>
+      <c r="D34" s="86"/>
+      <c r="E34" s="86"/>
+      <c r="F34" s="86"/>
+      <c r="G34" s="86"/>
+      <c r="H34" s="86"/>
+      <c r="I34" s="87"/>
+      <c r="J34" s="82"/>
+      <c r="K34" s="82"/>
+      <c r="L34" s="82"/>
+      <c r="M34" s="82"/>
+      <c r="N34" s="82"/>
+      <c r="O34" s="82"/>
+      <c r="P34" s="87"/>
+      <c r="Q34" s="82"/>
+      <c r="R34" s="82"/>
+    </row>
+    <row r="35" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A35" s="49"/>
+      <c r="B35" s="49"/>
+      <c r="C35" s="49"/>
+      <c r="D35" s="68"/>
+      <c r="E35" s="49"/>
+      <c r="F35" s="49"/>
+      <c r="G35" s="49"/>
+      <c r="H35" s="49"/>
+      <c r="I35" s="49"/>
+      <c r="J35" s="49"/>
+      <c r="K35" s="49"/>
+      <c r="L35" s="49"/>
+      <c r="M35" s="68"/>
+      <c r="N35" s="49"/>
+      <c r="O35" s="49"/>
+      <c r="P35" s="49"/>
+      <c r="Q35" s="49"/>
+      <c r="R35" s="49"/>
+    </row>
+    <row r="36" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A36" s="49"/>
+      <c r="B36" s="49"/>
+      <c r="C36" s="49"/>
+      <c r="D36" s="49"/>
+      <c r="E36" s="49"/>
+      <c r="F36" s="49"/>
+      <c r="G36" s="49"/>
+      <c r="H36" s="49"/>
+      <c r="I36" s="49"/>
+      <c r="J36" s="49"/>
+      <c r="K36" s="68"/>
+      <c r="L36" s="68"/>
+      <c r="M36" s="49"/>
+      <c r="N36" s="49"/>
+      <c r="O36" s="49"/>
+      <c r="P36" s="49"/>
+      <c r="Q36" s="49"/>
+      <c r="R36" s="49"/>
+    </row>
+  </sheetData>
+  <mergeCells count="18">
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="Q22:R22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="G23:H23"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="L23:M23"/>
+    <mergeCell ref="N23:O23"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="A22:A24"/>
+    <mergeCell ref="B22:B24"/>
+    <mergeCell ref="C22:H22"/>
+    <mergeCell ref="J22:O22"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{157A37C1-F88E-4B59-8842-1397A083790A}">
+  <dimension ref="A1:I33"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="27.140625" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" customWidth="1"/>
+    <col min="3" max="3" width="23.7109375" customWidth="1"/>
+    <col min="4" max="4" width="19.7109375" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" customWidth="1"/>
+    <col min="6" max="6" width="21.140625" customWidth="1"/>
+    <col min="7" max="7" width="17" customWidth="1"/>
+    <col min="8" max="8" width="20.42578125" customWidth="1"/>
+    <col min="9" max="9" width="20.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="39.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="102" t="s">
+        <v>71</v>
+      </c>
+      <c r="B1" s="103" t="s">
+        <v>72</v>
+      </c>
+      <c r="C1" s="103" t="s">
+        <v>73</v>
+      </c>
+      <c r="D1" s="103" t="s">
+        <v>74</v>
+      </c>
+      <c r="E1" s="103" t="s">
+        <v>75</v>
+      </c>
+      <c r="F1" s="103" t="s">
+        <v>76</v>
+      </c>
+      <c r="G1" s="103" t="s">
+        <v>77</v>
+      </c>
+      <c r="H1" s="103" t="s">
+        <v>78</v>
+      </c>
+      <c r="I1" s="104" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="105"/>
+      <c r="B2" s="106"/>
+      <c r="C2" s="107"/>
+      <c r="D2" s="108"/>
+      <c r="E2" s="106"/>
+      <c r="F2" s="106"/>
+      <c r="G2" s="106"/>
+      <c r="H2" s="109"/>
+      <c r="I2" s="110"/>
+    </row>
+    <row r="3" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="111"/>
+      <c r="B3" s="112"/>
+      <c r="C3" s="113"/>
+      <c r="D3" s="114"/>
+      <c r="E3" s="112"/>
+      <c r="F3" s="112"/>
+      <c r="G3" s="112"/>
+      <c r="H3" s="115"/>
+      <c r="I3" s="116"/>
+    </row>
+    <row r="4" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="105"/>
+      <c r="B4" s="106"/>
+      <c r="C4" s="107"/>
+      <c r="D4" s="108"/>
+      <c r="E4" s="106"/>
+      <c r="F4" s="106"/>
+      <c r="G4" s="106"/>
+      <c r="H4" s="109"/>
+      <c r="I4" s="110"/>
+    </row>
+    <row r="5" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="111"/>
+      <c r="B5" s="112"/>
+      <c r="C5" s="113"/>
+      <c r="D5" s="114"/>
+      <c r="E5" s="112"/>
+      <c r="F5" s="112"/>
+      <c r="G5" s="112"/>
+      <c r="H5" s="115"/>
+      <c r="I5" s="116"/>
+    </row>
+    <row r="6" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="105"/>
+      <c r="B6" s="106"/>
+      <c r="C6" s="107"/>
+      <c r="D6" s="108"/>
+      <c r="E6" s="106"/>
+      <c r="F6" s="106"/>
+      <c r="G6" s="106"/>
+      <c r="H6" s="109"/>
+      <c r="I6" s="117"/>
+    </row>
+    <row r="7" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="111"/>
+      <c r="B7" s="112"/>
+      <c r="C7" s="113"/>
+      <c r="D7" s="114"/>
+      <c r="E7" s="112"/>
+      <c r="F7" s="112"/>
+      <c r="G7" s="112"/>
+      <c r="H7" s="115"/>
+      <c r="I7" s="118"/>
+    </row>
+    <row r="8" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="105"/>
+      <c r="B8" s="106"/>
+      <c r="C8" s="107"/>
+      <c r="D8" s="108"/>
+      <c r="E8" s="106"/>
+      <c r="F8" s="106"/>
+      <c r="G8" s="106"/>
+      <c r="H8" s="109"/>
+      <c r="I8" s="117"/>
+    </row>
+    <row r="9" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="111"/>
+      <c r="B9" s="112"/>
+      <c r="C9" s="113"/>
+      <c r="D9" s="114"/>
+      <c r="E9" s="112"/>
+      <c r="F9" s="112"/>
+      <c r="G9" s="112"/>
+      <c r="H9" s="115"/>
+      <c r="I9" s="119"/>
+    </row>
+    <row r="10" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="105"/>
+      <c r="B10" s="106"/>
+      <c r="C10" s="107"/>
+      <c r="D10" s="108"/>
+      <c r="E10" s="106"/>
+      <c r="F10" s="106"/>
+      <c r="G10" s="106"/>
+      <c r="H10" s="109"/>
+      <c r="I10" s="120"/>
+    </row>
+    <row r="11" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="111"/>
+      <c r="B11" s="112"/>
+      <c r="C11" s="113"/>
+      <c r="D11" s="114"/>
+      <c r="E11" s="112"/>
+      <c r="F11" s="112"/>
+      <c r="G11" s="112"/>
+      <c r="H11" s="115"/>
+      <c r="I11" s="121"/>
+    </row>
+    <row r="12" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="105"/>
+      <c r="B12" s="106"/>
+      <c r="C12" s="107"/>
+      <c r="D12" s="106"/>
+      <c r="E12" s="106"/>
+      <c r="F12" s="106"/>
+      <c r="G12" s="106"/>
+      <c r="H12" s="109"/>
+      <c r="I12" s="120"/>
+    </row>
+    <row r="13" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="111"/>
+      <c r="B13" s="112"/>
+      <c r="C13" s="113"/>
+      <c r="D13" s="112"/>
+      <c r="E13" s="112"/>
+      <c r="F13" s="112"/>
+      <c r="G13" s="112"/>
+      <c r="H13" s="115"/>
+      <c r="I13" s="121"/>
+    </row>
+    <row r="14" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="105"/>
+      <c r="B14" s="106"/>
+      <c r="C14" s="107"/>
+      <c r="D14" s="106"/>
+      <c r="E14" s="106"/>
+      <c r="F14" s="106"/>
+      <c r="G14" s="106"/>
+      <c r="H14" s="109"/>
+      <c r="I14" s="120"/>
+    </row>
+    <row r="15" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="111"/>
+      <c r="B15" s="112"/>
+      <c r="C15" s="113"/>
+      <c r="D15" s="112"/>
+      <c r="E15" s="112"/>
+      <c r="F15" s="112"/>
+      <c r="G15" s="112"/>
+      <c r="H15" s="115"/>
+      <c r="I15" s="121"/>
+    </row>
+    <row r="16" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="105"/>
+      <c r="B16" s="106"/>
+      <c r="C16" s="107"/>
+      <c r="D16" s="106"/>
+      <c r="E16" s="106"/>
+      <c r="F16" s="106"/>
+      <c r="G16" s="106"/>
+      <c r="H16" s="109"/>
+      <c r="I16" s="120"/>
+    </row>
+    <row r="17" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="111"/>
+      <c r="B17" s="112"/>
+      <c r="C17" s="113"/>
+      <c r="D17" s="114"/>
+      <c r="E17" s="112"/>
+      <c r="F17" s="112"/>
+      <c r="G17" s="112"/>
+      <c r="H17" s="115"/>
+      <c r="I17" s="121"/>
+    </row>
+    <row r="18" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="105"/>
+      <c r="B18" s="106"/>
+      <c r="C18" s="106"/>
+      <c r="D18" s="106"/>
+      <c r="E18" s="106"/>
+      <c r="F18" s="106"/>
+      <c r="G18" s="106"/>
+      <c r="H18" s="109"/>
+      <c r="I18" s="110"/>
+    </row>
+    <row r="19" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="111"/>
+      <c r="B19" s="112"/>
+      <c r="C19" s="113"/>
+      <c r="D19" s="112"/>
+      <c r="E19" s="112"/>
+      <c r="F19" s="112"/>
+      <c r="G19" s="112"/>
+      <c r="H19" s="115"/>
+      <c r="I19" s="121"/>
+    </row>
+    <row r="20" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="105"/>
+      <c r="B20" s="106"/>
+      <c r="C20" s="107"/>
+      <c r="D20" s="106"/>
+      <c r="E20" s="106"/>
+      <c r="F20" s="106"/>
+      <c r="G20" s="106"/>
+      <c r="H20" s="109"/>
+      <c r="I20" s="120"/>
+    </row>
+    <row r="21" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="111"/>
+      <c r="B21" s="112"/>
+      <c r="C21" s="113"/>
+      <c r="D21" s="112"/>
+      <c r="E21" s="112"/>
+      <c r="F21" s="112"/>
+      <c r="G21" s="112"/>
+      <c r="H21" s="115"/>
+      <c r="I21" s="121"/>
+    </row>
+    <row r="22" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="105"/>
+      <c r="B22" s="106"/>
+      <c r="C22" s="107"/>
+      <c r="D22" s="106"/>
+      <c r="E22" s="106"/>
+      <c r="F22" s="106"/>
+      <c r="G22" s="106"/>
+      <c r="H22" s="109"/>
+      <c r="I22" s="117"/>
+    </row>
+    <row r="23" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="111"/>
+      <c r="B23" s="112"/>
+      <c r="C23" s="113"/>
+      <c r="D23" s="112"/>
+      <c r="E23" s="112"/>
+      <c r="F23" s="112"/>
+      <c r="G23" s="112"/>
+      <c r="H23" s="115"/>
+      <c r="I23" s="118"/>
+    </row>
+    <row r="24" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="105"/>
+      <c r="B24" s="106"/>
+      <c r="C24" s="107"/>
+      <c r="D24" s="106"/>
+      <c r="E24" s="106"/>
+      <c r="F24" s="106"/>
+      <c r="G24" s="106"/>
+      <c r="H24" s="109"/>
+      <c r="I24" s="117"/>
+    </row>
+    <row r="25" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="111"/>
+      <c r="B25" s="112"/>
+      <c r="C25" s="113"/>
+      <c r="D25" s="112"/>
+      <c r="E25" s="112"/>
+      <c r="F25" s="112"/>
+      <c r="G25" s="112"/>
+      <c r="H25" s="115"/>
+      <c r="I25" s="118"/>
+    </row>
+    <row r="26" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="105"/>
+      <c r="B26" s="106"/>
+      <c r="C26" s="107"/>
+      <c r="D26" s="106"/>
+      <c r="E26" s="106"/>
+      <c r="F26" s="106"/>
+      <c r="G26" s="106"/>
+      <c r="H26" s="109"/>
+      <c r="I26" s="117"/>
+    </row>
+    <row r="27" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="111"/>
+      <c r="B27" s="112"/>
+      <c r="C27" s="113"/>
+      <c r="D27" s="112"/>
+      <c r="E27" s="112"/>
+      <c r="F27" s="112"/>
+      <c r="G27" s="112"/>
+      <c r="H27" s="115"/>
+      <c r="I27" s="118"/>
+    </row>
+    <row r="28" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="105"/>
+      <c r="B28" s="106"/>
+      <c r="C28" s="107"/>
+      <c r="D28" s="106"/>
+      <c r="E28" s="106"/>
+      <c r="F28" s="106"/>
+      <c r="G28" s="106"/>
+      <c r="H28" s="109"/>
+      <c r="I28" s="117"/>
+    </row>
+    <row r="29" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="111"/>
+      <c r="B29" s="112"/>
+      <c r="C29" s="113"/>
+      <c r="D29" s="112"/>
+      <c r="E29" s="112"/>
+      <c r="F29" s="112"/>
+      <c r="G29" s="112"/>
+      <c r="H29" s="115"/>
+      <c r="I29" s="118"/>
+    </row>
+    <row r="30" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="105"/>
+      <c r="B30" s="106"/>
+      <c r="C30" s="107"/>
+      <c r="D30" s="106"/>
+      <c r="E30" s="106"/>
+      <c r="F30" s="106"/>
+      <c r="G30" s="106"/>
+      <c r="H30" s="109"/>
+      <c r="I30" s="117"/>
+    </row>
+    <row r="31" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="111"/>
+      <c r="B31" s="112"/>
+      <c r="C31" s="113"/>
+      <c r="D31" s="112"/>
+      <c r="E31" s="112"/>
+      <c r="F31" s="112"/>
+      <c r="G31" s="112"/>
+      <c r="H31" s="115"/>
+      <c r="I31" s="118"/>
+    </row>
+    <row r="32" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="105"/>
+      <c r="B32" s="106"/>
+      <c r="C32" s="107"/>
+      <c r="D32" s="106"/>
+      <c r="E32" s="106"/>
+      <c r="F32" s="106"/>
+      <c r="G32" s="106"/>
+      <c r="H32" s="122"/>
+      <c r="I32" s="117"/>
+    </row>
+    <row r="33" spans="1:9" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="123"/>
+      <c r="B33" s="124"/>
+      <c r="C33" s="124"/>
+      <c r="D33" s="124"/>
+      <c r="E33" s="124"/>
+      <c r="F33" s="124"/>
+      <c r="G33" s="124"/>
+      <c r="H33" s="124"/>
+      <c r="I33" s="119"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Extension Manual Input Added
</commit_message>
<xml_diff>
--- a/backend/utils/template2.xlsx
+++ b/backend/utils/template2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\My Stuff\Github\IPCR_GENERATOR-Thesis\backend\utils\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24C815B8-D821-4F73-A174-A65654E4106F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D21EDC5-F16B-40D5-B394-548954DB5318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -396,7 +396,7 @@
     <numFmt numFmtId="165" formatCode="mmmm\ d\,\ yyyy"/>
     <numFmt numFmtId="166" formatCode="mmmm\ dd\,\ yyyy"/>
   </numFmts>
-  <fonts count="41" x14ac:knownFonts="1">
+  <fonts count="42" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -533,6 +533,7 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -634,6 +635,14 @@
       <sz val="10"/>
       <color rgb="FF434343"/>
       <name val="Poppins"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="19">
@@ -1121,7 +1130,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="161">
+  <cellXfs count="162">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1293,9 +1302,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1493,6 +1499,63 @@
     <xf numFmtId="0" fontId="34" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="14" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="14" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1511,65 +1574,8 @@
     <xf numFmtId="0" fontId="31" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="13" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="13" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="14" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="14" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1592,6 +1598,12 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1874,16 +1886,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="102.75" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="153" t="s">
+      <c r="A1" s="152" t="s">
         <v>80</v>
       </c>
-      <c r="B1" s="154"/>
-      <c r="C1" s="154"/>
-      <c r="D1" s="154"/>
-      <c r="E1" s="154"/>
-      <c r="F1" s="154"/>
-      <c r="G1" s="154"/>
-      <c r="H1" s="154"/>
+      <c r="B1" s="153"/>
+      <c r="C1" s="153"/>
+      <c r="D1" s="153"/>
+      <c r="E1" s="153"/>
+      <c r="F1" s="153"/>
+      <c r="G1" s="153"/>
+      <c r="H1" s="153"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
     </row>
@@ -2430,16 +2442,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="102.75" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="153" t="s">
+      <c r="A1" s="152" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="154"/>
-      <c r="C1" s="154"/>
-      <c r="D1" s="154"/>
-      <c r="E1" s="154"/>
-      <c r="F1" s="154"/>
-      <c r="G1" s="154"/>
-      <c r="H1" s="154"/>
+      <c r="B1" s="153"/>
+      <c r="C1" s="153"/>
+      <c r="D1" s="153"/>
+      <c r="E1" s="153"/>
+      <c r="F1" s="153"/>
+      <c r="G1" s="153"/>
+      <c r="H1" s="153"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
     </row>
@@ -2990,16 +3002,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="102.75" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="153" t="s">
+      <c r="A1" s="152" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="154"/>
-      <c r="C1" s="154"/>
-      <c r="D1" s="154"/>
-      <c r="E1" s="154"/>
-      <c r="F1" s="154"/>
-      <c r="G1" s="154"/>
-      <c r="H1" s="154"/>
+      <c r="B1" s="153"/>
+      <c r="C1" s="153"/>
+      <c r="D1" s="153"/>
+      <c r="E1" s="153"/>
+      <c r="F1" s="153"/>
+      <c r="G1" s="153"/>
+      <c r="H1" s="153"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
     </row>
@@ -3550,16 +3562,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="102.75" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="153" t="s">
+      <c r="A1" s="152" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="154"/>
-      <c r="C1" s="154"/>
-      <c r="D1" s="154"/>
-      <c r="E1" s="154"/>
-      <c r="F1" s="154"/>
-      <c r="G1" s="154"/>
-      <c r="H1" s="154"/>
+      <c r="B1" s="153"/>
+      <c r="C1" s="153"/>
+      <c r="D1" s="153"/>
+      <c r="E1" s="153"/>
+      <c r="F1" s="153"/>
+      <c r="G1" s="153"/>
+      <c r="H1" s="153"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
     </row>
@@ -4121,35 +4133,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:30" ht="29.25" thickBot="1" x14ac:dyDescent="0.85">
-      <c r="A1" s="146" t="s">
+      <c r="A1" s="126" t="s">
         <v>46</v>
       </c>
-      <c r="B1" s="147"/>
-      <c r="C1" s="147"/>
-      <c r="D1" s="147"/>
-      <c r="E1" s="147"/>
-      <c r="F1" s="147"/>
-      <c r="G1" s="147"/>
-      <c r="H1" s="147"/>
-      <c r="I1" s="147"/>
-      <c r="J1" s="147"/>
-      <c r="K1" s="147"/>
-      <c r="L1" s="148"/>
+      <c r="B1" s="127"/>
+      <c r="C1" s="127"/>
+      <c r="D1" s="127"/>
+      <c r="E1" s="127"/>
+      <c r="F1" s="127"/>
+      <c r="G1" s="127"/>
+      <c r="H1" s="127"/>
+      <c r="I1" s="127"/>
+      <c r="J1" s="127"/>
+      <c r="K1" s="127"/>
+      <c r="L1" s="128"/>
       <c r="M1" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:30" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A2" s="88" t="s">
+      <c r="A2" s="87" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="89"/>
-      <c r="C2" s="158" t="s">
+      <c r="B2" s="88"/>
+      <c r="C2" s="157" t="s">
         <v>49</v>
       </c>
-      <c r="D2" s="159"/>
-      <c r="E2" s="160"/>
-      <c r="F2" s="90"/>
+      <c r="D2" s="158"/>
+      <c r="E2" s="159"/>
+      <c r="F2" s="89"/>
       <c r="G2" s="49"/>
       <c r="H2" s="49"/>
       <c r="I2" s="49"/>
@@ -4158,16 +4170,16 @@
       <c r="L2" s="49"/>
     </row>
     <row r="3" spans="1:30" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A3" s="88" t="s">
+      <c r="A3" s="87" t="s">
         <v>50</v>
       </c>
-      <c r="B3" s="91"/>
-      <c r="C3" s="158" t="s">
+      <c r="B3" s="90"/>
+      <c r="C3" s="157" t="s">
         <v>51</v>
       </c>
-      <c r="D3" s="159"/>
-      <c r="E3" s="160"/>
-      <c r="F3" s="89"/>
+      <c r="D3" s="158"/>
+      <c r="E3" s="159"/>
+      <c r="F3" s="88"/>
       <c r="G3" s="49"/>
       <c r="H3" s="49"/>
       <c r="I3" s="49"/>
@@ -4176,16 +4188,16 @@
       <c r="L3" s="49"/>
     </row>
     <row r="4" spans="1:30" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A4" s="88" t="s">
+      <c r="A4" s="87" t="s">
         <v>52</v>
       </c>
-      <c r="B4" s="91"/>
-      <c r="C4" s="158" t="s">
+      <c r="B4" s="90"/>
+      <c r="C4" s="157" t="s">
         <v>53</v>
       </c>
-      <c r="D4" s="159"/>
-      <c r="E4" s="160"/>
-      <c r="F4" s="89"/>
+      <c r="D4" s="158"/>
+      <c r="E4" s="159"/>
+      <c r="F4" s="88"/>
       <c r="G4" s="49"/>
       <c r="H4" s="49"/>
       <c r="I4" s="49"/>
@@ -4194,133 +4206,133 @@
       <c r="L4" s="49"/>
     </row>
     <row r="5" spans="1:30" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="92"/>
-      <c r="B5" s="92"/>
-      <c r="C5" s="92"/>
-      <c r="D5" s="92"/>
+      <c r="A5" s="91"/>
+      <c r="B5" s="91"/>
+      <c r="C5" s="91"/>
+      <c r="D5" s="91"/>
       <c r="E5" s="58"/>
       <c r="F5" s="58"/>
-      <c r="G5" s="92"/>
-      <c r="H5" s="92"/>
-      <c r="I5" s="92"/>
-      <c r="J5" s="92"/>
+      <c r="G5" s="91"/>
+      <c r="H5" s="91"/>
+      <c r="I5" s="91"/>
+      <c r="J5" s="91"/>
       <c r="K5" s="49"/>
       <c r="L5" s="49"/>
     </row>
     <row r="6" spans="1:30" ht="41.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="93" t="s">
+      <c r="A6" s="92" t="s">
         <v>54</v>
       </c>
-      <c r="B6" s="94"/>
-      <c r="C6" s="94"/>
-      <c r="D6" s="94"/>
-      <c r="E6" s="94"/>
-      <c r="F6" s="94"/>
-      <c r="G6" s="94"/>
-      <c r="H6" s="94"/>
-      <c r="I6" s="94"/>
-      <c r="J6" s="94"/>
+      <c r="B6" s="93"/>
+      <c r="C6" s="93"/>
+      <c r="D6" s="93"/>
+      <c r="E6" s="93"/>
+      <c r="F6" s="93"/>
+      <c r="G6" s="93"/>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="93"/>
       <c r="K6" s="49"/>
       <c r="L6" s="49"/>
-      <c r="U6" s="154"/>
-      <c r="V6" s="154"/>
+      <c r="U6" s="153"/>
+      <c r="V6" s="153"/>
     </row>
     <row r="7" spans="1:30" ht="67.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="95" t="s">
+      <c r="A7" s="94" t="s">
         <v>55</v>
       </c>
-      <c r="B7" s="125"/>
-      <c r="C7" s="125"/>
-      <c r="D7" s="125"/>
-      <c r="E7" s="125"/>
-      <c r="F7" s="125"/>
-      <c r="G7" s="125"/>
-      <c r="H7" s="125"/>
-      <c r="I7" s="125"/>
-      <c r="J7" s="125"/>
+      <c r="B7" s="124"/>
+      <c r="C7" s="124"/>
+      <c r="D7" s="124"/>
+      <c r="E7" s="124"/>
+      <c r="F7" s="124"/>
+      <c r="G7" s="124"/>
+      <c r="H7" s="124"/>
+      <c r="I7" s="124"/>
+      <c r="J7" s="124"/>
       <c r="K7" s="49"/>
       <c r="L7" s="49"/>
-      <c r="U7" s="154"/>
-      <c r="V7" s="154"/>
+      <c r="U7" s="153"/>
+      <c r="V7" s="153"/>
     </row>
     <row r="8" spans="1:30" ht="49.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="A8" s="95" t="s">
+      <c r="A8" s="94" t="s">
         <v>56</v>
       </c>
-      <c r="B8" s="125"/>
-      <c r="C8" s="126"/>
-      <c r="D8" s="125"/>
-      <c r="E8" s="125"/>
-      <c r="F8" s="126"/>
-      <c r="G8" s="125"/>
-      <c r="H8" s="126"/>
-      <c r="I8" s="125"/>
-      <c r="J8" s="125"/>
-      <c r="K8" s="96"/>
+      <c r="B8" s="124"/>
+      <c r="C8" s="125"/>
+      <c r="D8" s="124"/>
+      <c r="E8" s="124"/>
+      <c r="F8" s="125"/>
+      <c r="G8" s="124"/>
+      <c r="H8" s="125"/>
+      <c r="I8" s="124"/>
+      <c r="J8" s="124"/>
+      <c r="K8" s="95"/>
       <c r="L8" s="49"/>
     </row>
     <row r="9" spans="1:30" ht="41.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="A9" s="95" t="s">
+      <c r="A9" s="94" t="s">
         <v>57</v>
       </c>
-      <c r="B9" s="125"/>
-      <c r="C9" s="125"/>
-      <c r="D9" s="126"/>
-      <c r="E9" s="125"/>
-      <c r="F9" s="125"/>
-      <c r="G9" s="125"/>
-      <c r="H9" s="125"/>
-      <c r="I9" s="125"/>
-      <c r="J9" s="125"/>
-      <c r="K9" s="96"/>
+      <c r="B9" s="124"/>
+      <c r="C9" s="124"/>
+      <c r="D9" s="125"/>
+      <c r="E9" s="124"/>
+      <c r="F9" s="124"/>
+      <c r="G9" s="124"/>
+      <c r="H9" s="124"/>
+      <c r="I9" s="124"/>
+      <c r="J9" s="124"/>
+      <c r="K9" s="95"/>
       <c r="L9" s="49"/>
     </row>
     <row r="10" spans="1:30" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="A10" s="95" t="s">
+      <c r="A10" s="94" t="s">
         <v>58</v>
       </c>
-      <c r="B10" s="126"/>
-      <c r="C10" s="125"/>
-      <c r="D10" s="126"/>
-      <c r="E10" s="126"/>
-      <c r="F10" s="125"/>
-      <c r="G10" s="125"/>
-      <c r="H10" s="125"/>
-      <c r="I10" s="125"/>
-      <c r="J10" s="126"/>
-      <c r="K10" s="96"/>
+      <c r="B10" s="125"/>
+      <c r="C10" s="124"/>
+      <c r="D10" s="125"/>
+      <c r="E10" s="125"/>
+      <c r="F10" s="124"/>
+      <c r="G10" s="124"/>
+      <c r="H10" s="124"/>
+      <c r="I10" s="124"/>
+      <c r="J10" s="125"/>
+      <c r="K10" s="95"/>
       <c r="L10" s="49"/>
     </row>
     <row r="11" spans="1:30" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="A11" s="95" t="s">
+      <c r="A11" s="94" t="s">
         <v>59</v>
       </c>
-      <c r="B11" s="125"/>
-      <c r="C11" s="125"/>
-      <c r="D11" s="125"/>
-      <c r="E11" s="125"/>
-      <c r="F11" s="125"/>
-      <c r="G11" s="125"/>
-      <c r="H11" s="125"/>
-      <c r="I11" s="125"/>
-      <c r="J11" s="125"/>
-      <c r="K11" s="96"/>
+      <c r="B11" s="124"/>
+      <c r="C11" s="124"/>
+      <c r="D11" s="124"/>
+      <c r="E11" s="124"/>
+      <c r="F11" s="124"/>
+      <c r="G11" s="124"/>
+      <c r="H11" s="124"/>
+      <c r="I11" s="124"/>
+      <c r="J11" s="124"/>
+      <c r="K11" s="95"/>
       <c r="L11" s="49"/>
     </row>
     <row r="12" spans="1:30" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="A12" s="95" t="s">
+      <c r="A12" s="94" t="s">
         <v>60</v>
       </c>
-      <c r="B12" s="125"/>
-      <c r="C12" s="125"/>
-      <c r="D12" s="125"/>
-      <c r="E12" s="125"/>
-      <c r="F12" s="125"/>
-      <c r="G12" s="125"/>
-      <c r="H12" s="125"/>
-      <c r="I12" s="125"/>
-      <c r="J12" s="125"/>
-      <c r="K12" s="96"/>
+      <c r="B12" s="124"/>
+      <c r="C12" s="124"/>
+      <c r="D12" s="124"/>
+      <c r="E12" s="124"/>
+      <c r="F12" s="124"/>
+      <c r="G12" s="124"/>
+      <c r="H12" s="124"/>
+      <c r="I12" s="124"/>
+      <c r="J12" s="124"/>
+      <c r="K12" s="95"/>
       <c r="L12" s="49"/>
     </row>
     <row r="13" spans="1:30" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
@@ -4362,14 +4374,14 @@
       <c r="AD14" s="49"/>
     </row>
     <row r="15" spans="1:30" ht="24" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A15" s="88" t="s">
+      <c r="A15" s="87" t="s">
         <v>61</v>
       </c>
-      <c r="B15" s="155" t="s">
+      <c r="B15" s="154" t="s">
         <v>62</v>
       </c>
-      <c r="C15" s="156"/>
-      <c r="D15" s="157"/>
+      <c r="C15" s="155"/>
+      <c r="D15" s="156"/>
       <c r="E15" s="49"/>
       <c r="F15" s="49"/>
       <c r="G15" s="49"/>
@@ -4385,14 +4397,14 @@
       <c r="AD15" s="49"/>
     </row>
     <row r="16" spans="1:30" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="97"/>
-      <c r="B16" s="98" t="s">
+      <c r="A16" s="96"/>
+      <c r="B16" s="97" t="s">
         <v>63</v>
       </c>
-      <c r="C16" s="98" t="s">
+      <c r="C16" s="97" t="s">
         <v>64</v>
       </c>
-      <c r="D16" s="98" t="s">
+      <c r="D16" s="97" t="s">
         <v>65</v>
       </c>
       <c r="E16" s="49"/>
@@ -4410,10 +4422,10 @@
       <c r="AD16" s="49"/>
     </row>
     <row r="17" spans="1:30" ht="24" thickBot="1" x14ac:dyDescent="0.7">
-      <c r="A17" s="97"/>
-      <c r="B17" s="99"/>
-      <c r="C17" s="99"/>
-      <c r="D17" s="99"/>
+      <c r="A17" s="96"/>
+      <c r="B17" s="98"/>
+      <c r="C17" s="98"/>
+      <c r="D17" s="98"/>
       <c r="E17" s="49"/>
       <c r="F17" s="49"/>
       <c r="G17" s="49"/>
@@ -4467,7 +4479,7 @@
       <c r="AD19" s="49"/>
     </row>
     <row r="20" spans="1:30" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A20" s="100" t="s">
+      <c r="A20" s="99" t="s">
         <v>66</v>
       </c>
       <c r="B20" s="49"/>
@@ -4488,10 +4500,10 @@
       <c r="AD20" s="49"/>
     </row>
     <row r="21" spans="1:30" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A21" s="67" t="s">
+      <c r="A21" s="66" t="s">
         <v>67</v>
       </c>
-      <c r="B21" s="101"/>
+      <c r="B21" s="100"/>
       <c r="C21" s="49"/>
       <c r="D21" s="49"/>
       <c r="E21" s="49"/>
@@ -4509,10 +4521,10 @@
       <c r="AD21" s="49"/>
     </row>
     <row r="22" spans="1:30" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A22" s="67" t="s">
+      <c r="A22" s="66" t="s">
         <v>68</v>
       </c>
-      <c r="B22" s="101"/>
+      <c r="B22" s="100"/>
       <c r="C22" s="49"/>
       <c r="D22" s="49"/>
       <c r="E22" s="49"/>
@@ -4530,10 +4542,10 @@
       <c r="AD22" s="49"/>
     </row>
     <row r="23" spans="1:30" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A23" s="67" t="s">
+      <c r="A23" s="66" t="s">
         <v>69</v>
       </c>
-      <c r="B23" s="101"/>
+      <c r="B23" s="100"/>
       <c r="C23" s="49"/>
       <c r="D23" s="49"/>
       <c r="E23" s="49"/>
@@ -4551,10 +4563,10 @@
       <c r="AD23" s="49"/>
     </row>
     <row r="24" spans="1:30" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A24" s="67" t="s">
+      <c r="A24" s="66" t="s">
         <v>70</v>
       </c>
-      <c r="B24" s="101"/>
+      <c r="B24" s="100"/>
       <c r="C24" s="49"/>
       <c r="D24" s="49"/>
       <c r="E24" s="49"/>
@@ -4608,20 +4620,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="29.25" thickBot="1" x14ac:dyDescent="0.85">
-      <c r="A1" s="146" t="s">
+      <c r="A1" s="126" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="147"/>
-      <c r="C1" s="147"/>
-      <c r="D1" s="147"/>
-      <c r="E1" s="147"/>
-      <c r="F1" s="147"/>
-      <c r="G1" s="147"/>
-      <c r="H1" s="147"/>
-      <c r="I1" s="147"/>
-      <c r="J1" s="147"/>
-      <c r="K1" s="147"/>
-      <c r="L1" s="148"/>
+      <c r="B1" s="127"/>
+      <c r="C1" s="127"/>
+      <c r="D1" s="127"/>
+      <c r="E1" s="127"/>
+      <c r="F1" s="127"/>
+      <c r="G1" s="127"/>
+      <c r="H1" s="127"/>
+      <c r="I1" s="127"/>
+      <c r="J1" s="127"/>
+      <c r="K1" s="127"/>
+      <c r="L1" s="128"/>
       <c r="M1" s="49"/>
       <c r="N1" s="49"/>
       <c r="O1" s="49"/>
@@ -4630,10 +4642,10 @@
       <c r="R1" s="49"/>
     </row>
     <row r="2" spans="1:18" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.7">
-      <c r="A2" s="149" t="s">
+      <c r="A2" s="129" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="150"/>
+      <c r="B2" s="130"/>
       <c r="C2" s="50"/>
       <c r="D2" s="49"/>
       <c r="E2" s="49"/>
@@ -4698,22 +4710,22 @@
       <c r="B5" s="54" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="151" t="s">
+      <c r="C5" s="131" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="152"/>
-      <c r="E5" s="138" t="s">
+      <c r="D5" s="132"/>
+      <c r="E5" s="133" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="139"/>
-      <c r="G5" s="142" t="s">
+      <c r="F5" s="134"/>
+      <c r="G5" s="135" t="s">
         <v>18</v>
       </c>
-      <c r="H5" s="143"/>
-      <c r="I5" s="144" t="s">
+      <c r="H5" s="136"/>
+      <c r="I5" s="137" t="s">
         <v>19</v>
       </c>
-      <c r="J5" s="145"/>
+      <c r="J5" s="138"/>
       <c r="K5" s="54" t="s">
         <v>20</v>
       </c>
@@ -4763,23 +4775,23 @@
       <c r="Q6" s="55"/>
       <c r="R6" s="55"/>
     </row>
-    <row r="7" spans="1:18" ht="50.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A7" s="127" t="s">
+    <row r="7" spans="1:18" ht="50.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="145" t="s">
         <v>24</v>
       </c>
       <c r="B7" s="59" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="60"/>
-      <c r="D7" s="60"/>
-      <c r="E7" s="60"/>
-      <c r="F7" s="57"/>
-      <c r="G7" s="60"/>
-      <c r="H7" s="57"/>
-      <c r="I7" s="60"/>
-      <c r="J7" s="57"/>
-      <c r="K7" s="60"/>
-      <c r="L7" s="60"/>
+      <c r="C7" s="160"/>
+      <c r="D7" s="160"/>
+      <c r="E7" s="160"/>
+      <c r="F7" s="161"/>
+      <c r="G7" s="160"/>
+      <c r="H7" s="161"/>
+      <c r="I7" s="160"/>
+      <c r="J7" s="161"/>
+      <c r="K7" s="160"/>
+      <c r="L7" s="160"/>
       <c r="M7" s="49"/>
       <c r="N7" s="49"/>
       <c r="O7" s="49"/>
@@ -4788,20 +4800,20 @@
       <c r="R7" s="49"/>
     </row>
     <row r="8" spans="1:18" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A8" s="128"/>
-      <c r="B8" s="61" t="s">
+      <c r="A8" s="146"/>
+      <c r="B8" s="60" t="s">
         <v>26</v>
       </c>
-      <c r="C8" s="60"/>
-      <c r="D8" s="60"/>
-      <c r="E8" s="60"/>
-      <c r="F8" s="57"/>
-      <c r="G8" s="60"/>
-      <c r="H8" s="57"/>
-      <c r="I8" s="60"/>
-      <c r="J8" s="57"/>
-      <c r="K8" s="60"/>
-      <c r="L8" s="60"/>
+      <c r="C8" s="160"/>
+      <c r="D8" s="160"/>
+      <c r="E8" s="160"/>
+      <c r="F8" s="161"/>
+      <c r="G8" s="160"/>
+      <c r="H8" s="161"/>
+      <c r="I8" s="160"/>
+      <c r="J8" s="161"/>
+      <c r="K8" s="160"/>
+      <c r="L8" s="160"/>
       <c r="M8" s="49"/>
       <c r="N8" s="49"/>
       <c r="O8" s="49"/>
@@ -4810,20 +4822,20 @@
       <c r="R8" s="49"/>
     </row>
     <row r="9" spans="1:18" ht="39.75" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A9" s="129"/>
-      <c r="B9" s="61" t="s">
+      <c r="A9" s="147"/>
+      <c r="B9" s="60" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="60"/>
-      <c r="D9" s="60"/>
-      <c r="E9" s="60"/>
-      <c r="F9" s="57"/>
-      <c r="G9" s="60"/>
-      <c r="H9" s="57"/>
-      <c r="I9" s="60"/>
-      <c r="J9" s="57"/>
-      <c r="K9" s="60"/>
-      <c r="L9" s="60"/>
+      <c r="C9" s="160"/>
+      <c r="D9" s="160"/>
+      <c r="E9" s="160"/>
+      <c r="F9" s="161"/>
+      <c r="G9" s="160"/>
+      <c r="H9" s="161"/>
+      <c r="I9" s="160"/>
+      <c r="J9" s="161"/>
+      <c r="K9" s="160"/>
+      <c r="L9" s="160"/>
       <c r="M9" s="49"/>
       <c r="N9" s="49"/>
       <c r="O9" s="49"/>
@@ -4852,10 +4864,10 @@
       <c r="R10" s="49"/>
     </row>
     <row r="11" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A11" s="62" t="s">
+      <c r="A11" s="61" t="s">
         <v>28</v>
       </c>
-      <c r="B11" s="63"/>
+      <c r="B11" s="62"/>
       <c r="C11" s="49"/>
       <c r="D11" s="49"/>
       <c r="E11" s="49"/>
@@ -4874,10 +4886,10 @@
       <c r="R11" s="49"/>
     </row>
     <row r="12" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="64" t="s">
+      <c r="A12" s="63" t="s">
         <v>29</v>
       </c>
-      <c r="B12" s="63"/>
+      <c r="B12" s="62"/>
       <c r="C12" s="49"/>
       <c r="D12" s="49"/>
       <c r="E12" s="49"/>
@@ -4896,10 +4908,10 @@
       <c r="R12" s="49"/>
     </row>
     <row r="13" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="64" t="s">
+      <c r="A13" s="63" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="63"/>
+      <c r="B13" s="62"/>
       <c r="C13" s="49"/>
       <c r="D13" s="49"/>
       <c r="E13" s="49"/>
@@ -4938,20 +4950,20 @@
       <c r="R14" s="49"/>
     </row>
     <row r="15" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A15" s="66" t="s">
+      <c r="A15" s="65" t="s">
         <v>81</v>
       </c>
       <c r="B15" s="49"/>
-      <c r="C15" s="66" t="s">
+      <c r="C15" s="65" t="s">
         <v>31</v>
       </c>
       <c r="D15" s="49"/>
       <c r="E15" s="49"/>
-      <c r="F15" s="66" t="s">
+      <c r="F15" s="65" t="s">
         <v>32</v>
       </c>
       <c r="G15" s="49"/>
-      <c r="H15" s="66" t="s">
+      <c r="H15" s="65" t="s">
         <v>33</v>
       </c>
       <c r="I15" s="49"/>
@@ -4966,14 +4978,14 @@
       <c r="R15" s="49"/>
     </row>
     <row r="16" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A16" s="67"/>
+      <c r="A16" s="66"/>
       <c r="B16" s="49"/>
-      <c r="C16" s="67"/>
+      <c r="C16" s="66"/>
       <c r="D16" s="49"/>
       <c r="E16" s="49"/>
-      <c r="F16" s="67"/>
+      <c r="F16" s="66"/>
       <c r="G16" s="49"/>
-      <c r="H16" s="65"/>
+      <c r="H16" s="64"/>
       <c r="I16" s="49"/>
       <c r="J16" s="49"/>
       <c r="K16" s="49"/>
@@ -4986,21 +4998,21 @@
       <c r="R16" s="49"/>
     </row>
     <row r="17" spans="1:18" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A17" s="68"/>
-      <c r="B17" s="67" t="s">
+      <c r="A17" s="67"/>
+      <c r="B17" s="66" t="s">
         <v>34</v>
       </c>
-      <c r="C17" s="68"/>
-      <c r="D17" s="65" t="s">
+      <c r="C17" s="67"/>
+      <c r="D17" s="64" t="s">
         <v>34</v>
       </c>
       <c r="E17" s="49"/>
-      <c r="F17" s="68"/>
-      <c r="G17" s="65" t="s">
+      <c r="F17" s="67"/>
+      <c r="G17" s="64" t="s">
         <v>34</v>
       </c>
-      <c r="H17" s="68"/>
-      <c r="I17" s="65" t="s">
+      <c r="H17" s="67"/>
+      <c r="I17" s="64" t="s">
         <v>34</v>
       </c>
       <c r="J17" s="49"/>
@@ -5014,21 +5026,21 @@
       <c r="R17" s="49"/>
     </row>
     <row r="18" spans="1:18" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A18" s="68"/>
-      <c r="B18" s="67" t="s">
+      <c r="A18" s="67"/>
+      <c r="B18" s="66" t="s">
         <v>35</v>
       </c>
-      <c r="C18" s="68"/>
-      <c r="D18" s="65" t="s">
+      <c r="C18" s="67"/>
+      <c r="D18" s="64" t="s">
         <v>35</v>
       </c>
       <c r="E18" s="49"/>
-      <c r="F18" s="68"/>
-      <c r="G18" s="65" t="s">
+      <c r="F18" s="67"/>
+      <c r="G18" s="64" t="s">
         <v>35</v>
       </c>
-      <c r="H18" s="68"/>
-      <c r="I18" s="65" t="s">
+      <c r="H18" s="67"/>
+      <c r="I18" s="64" t="s">
         <v>35</v>
       </c>
       <c r="J18" s="49"/>
@@ -5042,21 +5054,21 @@
       <c r="R18" s="49"/>
     </row>
     <row r="19" spans="1:18" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A19" s="68"/>
-      <c r="B19" s="67" t="s">
+      <c r="A19" s="67"/>
+      <c r="B19" s="66" t="s">
         <v>36</v>
       </c>
-      <c r="C19" s="68"/>
-      <c r="D19" s="65" t="s">
+      <c r="C19" s="67"/>
+      <c r="D19" s="64" t="s">
         <v>36</v>
       </c>
       <c r="E19" s="49"/>
-      <c r="F19" s="68"/>
-      <c r="G19" s="65" t="s">
+      <c r="F19" s="67"/>
+      <c r="G19" s="64" t="s">
         <v>36</v>
       </c>
-      <c r="H19" s="68"/>
-      <c r="I19" s="65" t="s">
+      <c r="H19" s="67"/>
+      <c r="I19" s="64" t="s">
         <v>36</v>
       </c>
       <c r="J19" s="49"/>
@@ -5110,320 +5122,320 @@
       <c r="R21" s="52"/>
     </row>
     <row r="22" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A22" s="130" t="s">
+      <c r="A22" s="148" t="s">
         <v>37</v>
       </c>
-      <c r="B22" s="130" t="s">
+      <c r="B22" s="148" t="s">
         <v>38</v>
       </c>
-      <c r="C22" s="133" t="s">
+      <c r="C22" s="139" t="s">
         <v>39</v>
       </c>
-      <c r="D22" s="134"/>
-      <c r="E22" s="134"/>
-      <c r="F22" s="134"/>
-      <c r="G22" s="134"/>
-      <c r="H22" s="135"/>
+      <c r="D22" s="151"/>
+      <c r="E22" s="151"/>
+      <c r="F22" s="151"/>
+      <c r="G22" s="151"/>
+      <c r="H22" s="140"/>
       <c r="I22" s="57"/>
-      <c r="J22" s="133" t="s">
+      <c r="J22" s="139" t="s">
         <v>40</v>
       </c>
-      <c r="K22" s="134"/>
-      <c r="L22" s="134"/>
-      <c r="M22" s="134"/>
-      <c r="N22" s="134"/>
-      <c r="O22" s="135"/>
+      <c r="K22" s="151"/>
+      <c r="L22" s="151"/>
+      <c r="M22" s="151"/>
+      <c r="N22" s="151"/>
+      <c r="O22" s="140"/>
       <c r="P22" s="57"/>
-      <c r="Q22" s="133">
+      <c r="Q22" s="139">
         <v>2025</v>
       </c>
-      <c r="R22" s="135"/>
+      <c r="R22" s="140"/>
     </row>
     <row r="23" spans="1:18" ht="39.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="131"/>
-      <c r="B23" s="131"/>
-      <c r="C23" s="136" t="s">
+      <c r="A23" s="149"/>
+      <c r="B23" s="149"/>
+      <c r="C23" s="141" t="s">
         <v>41</v>
       </c>
-      <c r="D23" s="137"/>
-      <c r="E23" s="138" t="s">
+      <c r="D23" s="142"/>
+      <c r="E23" s="133" t="s">
         <v>42</v>
       </c>
-      <c r="F23" s="139"/>
-      <c r="G23" s="140" t="s">
+      <c r="F23" s="134"/>
+      <c r="G23" s="143" t="s">
         <v>39</v>
       </c>
-      <c r="H23" s="141"/>
+      <c r="H23" s="144"/>
       <c r="I23" s="58"/>
-      <c r="J23" s="142" t="s">
+      <c r="J23" s="135" t="s">
         <v>43</v>
       </c>
-      <c r="K23" s="143"/>
-      <c r="L23" s="144" t="s">
+      <c r="K23" s="136"/>
+      <c r="L23" s="137" t="s">
         <v>44</v>
       </c>
-      <c r="M23" s="145"/>
-      <c r="N23" s="140" t="s">
+      <c r="M23" s="138"/>
+      <c r="N23" s="143" t="s">
         <v>40</v>
       </c>
-      <c r="O23" s="141"/>
+      <c r="O23" s="144"/>
       <c r="P23" s="58"/>
-      <c r="Q23" s="69" t="s">
+      <c r="Q23" s="68" t="s">
         <v>20</v>
       </c>
-      <c r="R23" s="69" t="s">
+      <c r="R23" s="68" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="24" spans="1:18" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="132"/>
-      <c r="B24" s="132"/>
-      <c r="C24" s="70" t="s">
+      <c r="A24" s="150"/>
+      <c r="B24" s="150"/>
+      <c r="C24" s="69" t="s">
         <v>22</v>
       </c>
-      <c r="D24" s="71" t="s">
+      <c r="D24" s="70" t="s">
         <v>45</v>
       </c>
-      <c r="E24" s="70" t="s">
+      <c r="E24" s="69" t="s">
         <v>22</v>
       </c>
-      <c r="F24" s="72" t="s">
+      <c r="F24" s="71" t="s">
         <v>45</v>
       </c>
-      <c r="G24" s="73" t="s">
+      <c r="G24" s="72" t="s">
         <v>22</v>
       </c>
-      <c r="H24" s="73" t="s">
+      <c r="H24" s="72" t="s">
         <v>45</v>
       </c>
       <c r="I24" s="58"/>
-      <c r="J24" s="70" t="s">
+      <c r="J24" s="69" t="s">
         <v>22</v>
       </c>
-      <c r="K24" s="74" t="s">
+      <c r="K24" s="73" t="s">
         <v>45</v>
       </c>
-      <c r="L24" s="70" t="s">
+      <c r="L24" s="69" t="s">
         <v>22</v>
       </c>
-      <c r="M24" s="75" t="s">
+      <c r="M24" s="74" t="s">
         <v>45</v>
       </c>
-      <c r="N24" s="73" t="s">
+      <c r="N24" s="72" t="s">
         <v>22</v>
       </c>
-      <c r="O24" s="73" t="s">
+      <c r="O24" s="72" t="s">
         <v>45</v>
       </c>
       <c r="P24" s="58"/>
-      <c r="Q24" s="76"/>
-      <c r="R24" s="76"/>
+      <c r="Q24" s="75"/>
+      <c r="R24" s="75"/>
     </row>
     <row r="25" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A25" s="77"/>
-      <c r="B25" s="78"/>
-      <c r="C25" s="79"/>
-      <c r="D25" s="80"/>
-      <c r="E25" s="79"/>
-      <c r="F25" s="81"/>
-      <c r="G25" s="82"/>
-      <c r="H25" s="82"/>
+      <c r="A25" s="76"/>
+      <c r="B25" s="77"/>
+      <c r="C25" s="78"/>
+      <c r="D25" s="79"/>
+      <c r="E25" s="78"/>
+      <c r="F25" s="80"/>
+      <c r="G25" s="81"/>
+      <c r="H25" s="81"/>
       <c r="I25" s="57"/>
-      <c r="J25" s="79"/>
-      <c r="K25" s="83"/>
-      <c r="L25" s="79"/>
-      <c r="M25" s="84"/>
-      <c r="N25" s="82"/>
-      <c r="O25" s="82"/>
+      <c r="J25" s="78"/>
+      <c r="K25" s="82"/>
+      <c r="L25" s="78"/>
+      <c r="M25" s="83"/>
+      <c r="N25" s="81"/>
+      <c r="O25" s="81"/>
       <c r="P25" s="57"/>
-      <c r="Q25" s="82"/>
-      <c r="R25" s="82"/>
+      <c r="Q25" s="81"/>
+      <c r="R25" s="81"/>
     </row>
     <row r="26" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A26" s="77"/>
-      <c r="B26" s="78"/>
-      <c r="C26" s="79"/>
-      <c r="D26" s="80"/>
-      <c r="E26" s="79"/>
-      <c r="F26" s="81"/>
-      <c r="G26" s="82"/>
-      <c r="H26" s="82"/>
+      <c r="A26" s="76"/>
+      <c r="B26" s="77"/>
+      <c r="C26" s="78"/>
+      <c r="D26" s="79"/>
+      <c r="E26" s="78"/>
+      <c r="F26" s="80"/>
+      <c r="G26" s="81"/>
+      <c r="H26" s="81"/>
       <c r="I26" s="57"/>
-      <c r="J26" s="79"/>
-      <c r="K26" s="83"/>
-      <c r="L26" s="79"/>
-      <c r="M26" s="84"/>
-      <c r="N26" s="82"/>
-      <c r="O26" s="82"/>
+      <c r="J26" s="78"/>
+      <c r="K26" s="82"/>
+      <c r="L26" s="78"/>
+      <c r="M26" s="83"/>
+      <c r="N26" s="81"/>
+      <c r="O26" s="81"/>
       <c r="P26" s="57"/>
-      <c r="Q26" s="82"/>
-      <c r="R26" s="82"/>
+      <c r="Q26" s="81"/>
+      <c r="R26" s="81"/>
     </row>
     <row r="27" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A27" s="77"/>
-      <c r="B27" s="78"/>
-      <c r="C27" s="79"/>
-      <c r="D27" s="80"/>
-      <c r="E27" s="79"/>
-      <c r="F27" s="81"/>
-      <c r="G27" s="82"/>
-      <c r="H27" s="82"/>
+      <c r="A27" s="76"/>
+      <c r="B27" s="77"/>
+      <c r="C27" s="78"/>
+      <c r="D27" s="79"/>
+      <c r="E27" s="78"/>
+      <c r="F27" s="80"/>
+      <c r="G27" s="81"/>
+      <c r="H27" s="81"/>
       <c r="I27" s="57"/>
-      <c r="J27" s="79"/>
-      <c r="K27" s="83"/>
-      <c r="L27" s="79"/>
-      <c r="M27" s="84"/>
-      <c r="N27" s="82"/>
-      <c r="O27" s="82"/>
+      <c r="J27" s="78"/>
+      <c r="K27" s="82"/>
+      <c r="L27" s="78"/>
+      <c r="M27" s="83"/>
+      <c r="N27" s="81"/>
+      <c r="O27" s="81"/>
       <c r="P27" s="57"/>
-      <c r="Q27" s="82"/>
-      <c r="R27" s="82"/>
+      <c r="Q27" s="81"/>
+      <c r="R27" s="81"/>
     </row>
     <row r="28" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A28" s="77"/>
-      <c r="B28" s="78"/>
-      <c r="C28" s="79"/>
-      <c r="D28" s="80"/>
-      <c r="E28" s="79"/>
-      <c r="F28" s="81"/>
-      <c r="G28" s="82"/>
-      <c r="H28" s="82"/>
+      <c r="A28" s="76"/>
+      <c r="B28" s="77"/>
+      <c r="C28" s="78"/>
+      <c r="D28" s="79"/>
+      <c r="E28" s="78"/>
+      <c r="F28" s="80"/>
+      <c r="G28" s="81"/>
+      <c r="H28" s="81"/>
       <c r="I28" s="57"/>
-      <c r="J28" s="79"/>
-      <c r="K28" s="83"/>
-      <c r="L28" s="79"/>
-      <c r="M28" s="84"/>
-      <c r="N28" s="82"/>
-      <c r="O28" s="82"/>
+      <c r="J28" s="78"/>
+      <c r="K28" s="82"/>
+      <c r="L28" s="78"/>
+      <c r="M28" s="83"/>
+      <c r="N28" s="81"/>
+      <c r="O28" s="81"/>
       <c r="P28" s="57"/>
-      <c r="Q28" s="82"/>
-      <c r="R28" s="82"/>
+      <c r="Q28" s="81"/>
+      <c r="R28" s="81"/>
     </row>
     <row r="29" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A29" s="77"/>
-      <c r="B29" s="78"/>
-      <c r="C29" s="79"/>
-      <c r="D29" s="80"/>
-      <c r="E29" s="79"/>
-      <c r="F29" s="81"/>
-      <c r="G29" s="82"/>
-      <c r="H29" s="82"/>
+      <c r="A29" s="76"/>
+      <c r="B29" s="77"/>
+      <c r="C29" s="78"/>
+      <c r="D29" s="79"/>
+      <c r="E29" s="78"/>
+      <c r="F29" s="80"/>
+      <c r="G29" s="81"/>
+      <c r="H29" s="81"/>
       <c r="I29" s="57"/>
-      <c r="J29" s="79"/>
-      <c r="K29" s="83"/>
-      <c r="L29" s="79"/>
-      <c r="M29" s="84"/>
-      <c r="N29" s="82"/>
-      <c r="O29" s="82"/>
+      <c r="J29" s="78"/>
+      <c r="K29" s="82"/>
+      <c r="L29" s="78"/>
+      <c r="M29" s="83"/>
+      <c r="N29" s="81"/>
+      <c r="O29" s="81"/>
       <c r="P29" s="57"/>
-      <c r="Q29" s="82"/>
-      <c r="R29" s="82"/>
+      <c r="Q29" s="81"/>
+      <c r="R29" s="81"/>
     </row>
     <row r="30" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A30" s="77"/>
-      <c r="B30" s="78"/>
-      <c r="C30" s="79"/>
-      <c r="D30" s="80"/>
-      <c r="E30" s="79"/>
-      <c r="F30" s="81"/>
-      <c r="G30" s="82"/>
-      <c r="H30" s="82"/>
+      <c r="A30" s="76"/>
+      <c r="B30" s="77"/>
+      <c r="C30" s="78"/>
+      <c r="D30" s="79"/>
+      <c r="E30" s="78"/>
+      <c r="F30" s="80"/>
+      <c r="G30" s="81"/>
+      <c r="H30" s="81"/>
       <c r="I30" s="57"/>
-      <c r="J30" s="79"/>
-      <c r="K30" s="83"/>
-      <c r="L30" s="79"/>
-      <c r="M30" s="84"/>
-      <c r="N30" s="82"/>
-      <c r="O30" s="82"/>
+      <c r="J30" s="78"/>
+      <c r="K30" s="82"/>
+      <c r="L30" s="78"/>
+      <c r="M30" s="83"/>
+      <c r="N30" s="81"/>
+      <c r="O30" s="81"/>
       <c r="P30" s="57"/>
-      <c r="Q30" s="82"/>
-      <c r="R30" s="82"/>
+      <c r="Q30" s="81"/>
+      <c r="R30" s="81"/>
     </row>
     <row r="31" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A31" s="77"/>
-      <c r="B31" s="78"/>
-      <c r="C31" s="79"/>
-      <c r="D31" s="80"/>
-      <c r="E31" s="79"/>
-      <c r="F31" s="81"/>
-      <c r="G31" s="82"/>
-      <c r="H31" s="82"/>
+      <c r="A31" s="76"/>
+      <c r="B31" s="77"/>
+      <c r="C31" s="78"/>
+      <c r="D31" s="79"/>
+      <c r="E31" s="78"/>
+      <c r="F31" s="80"/>
+      <c r="G31" s="81"/>
+      <c r="H31" s="81"/>
       <c r="I31" s="57"/>
-      <c r="J31" s="79"/>
-      <c r="K31" s="83"/>
-      <c r="L31" s="79"/>
-      <c r="M31" s="84"/>
-      <c r="N31" s="82"/>
-      <c r="O31" s="82"/>
+      <c r="J31" s="78"/>
+      <c r="K31" s="82"/>
+      <c r="L31" s="78"/>
+      <c r="M31" s="83"/>
+      <c r="N31" s="81"/>
+      <c r="O31" s="81"/>
       <c r="P31" s="57"/>
-      <c r="Q31" s="82"/>
-      <c r="R31" s="82"/>
+      <c r="Q31" s="81"/>
+      <c r="R31" s="81"/>
     </row>
     <row r="32" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A32" s="77"/>
-      <c r="B32" s="78"/>
-      <c r="C32" s="79"/>
-      <c r="D32" s="80"/>
-      <c r="E32" s="79"/>
-      <c r="F32" s="81"/>
-      <c r="G32" s="82"/>
-      <c r="H32" s="82"/>
+      <c r="A32" s="76"/>
+      <c r="B32" s="77"/>
+      <c r="C32" s="78"/>
+      <c r="D32" s="79"/>
+      <c r="E32" s="78"/>
+      <c r="F32" s="80"/>
+      <c r="G32" s="81"/>
+      <c r="H32" s="81"/>
       <c r="I32" s="57"/>
-      <c r="J32" s="79"/>
-      <c r="K32" s="83"/>
-      <c r="L32" s="79"/>
-      <c r="M32" s="84"/>
-      <c r="N32" s="82"/>
-      <c r="O32" s="82"/>
+      <c r="J32" s="78"/>
+      <c r="K32" s="82"/>
+      <c r="L32" s="78"/>
+      <c r="M32" s="83"/>
+      <c r="N32" s="81"/>
+      <c r="O32" s="81"/>
       <c r="P32" s="57"/>
-      <c r="Q32" s="82"/>
-      <c r="R32" s="82"/>
+      <c r="Q32" s="81"/>
+      <c r="R32" s="81"/>
     </row>
     <row r="33" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A33" s="77"/>
-      <c r="B33" s="78"/>
-      <c r="C33" s="79"/>
-      <c r="D33" s="80"/>
-      <c r="E33" s="79"/>
-      <c r="F33" s="81"/>
-      <c r="G33" s="82"/>
-      <c r="H33" s="82"/>
+      <c r="A33" s="76"/>
+      <c r="B33" s="77"/>
+      <c r="C33" s="78"/>
+      <c r="D33" s="79"/>
+      <c r="E33" s="78"/>
+      <c r="F33" s="80"/>
+      <c r="G33" s="81"/>
+      <c r="H33" s="81"/>
       <c r="I33" s="57"/>
-      <c r="J33" s="79"/>
-      <c r="K33" s="83"/>
-      <c r="L33" s="79"/>
-      <c r="M33" s="84"/>
-      <c r="N33" s="82"/>
-      <c r="O33" s="82"/>
+      <c r="J33" s="78"/>
+      <c r="K33" s="82"/>
+      <c r="L33" s="78"/>
+      <c r="M33" s="83"/>
+      <c r="N33" s="81"/>
+      <c r="O33" s="81"/>
       <c r="P33" s="57"/>
-      <c r="Q33" s="82"/>
-      <c r="R33" s="82"/>
+      <c r="Q33" s="81"/>
+      <c r="R33" s="81"/>
     </row>
     <row r="34" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A34" s="49"/>
-      <c r="B34" s="85"/>
-      <c r="C34" s="86"/>
-      <c r="D34" s="86"/>
-      <c r="E34" s="86"/>
-      <c r="F34" s="86"/>
-      <c r="G34" s="86"/>
-      <c r="H34" s="86"/>
-      <c r="I34" s="87"/>
-      <c r="J34" s="82"/>
-      <c r="K34" s="82"/>
-      <c r="L34" s="82"/>
-      <c r="M34" s="82"/>
-      <c r="N34" s="82"/>
-      <c r="O34" s="82"/>
-      <c r="P34" s="87"/>
-      <c r="Q34" s="82"/>
-      <c r="R34" s="82"/>
+      <c r="B34" s="84"/>
+      <c r="C34" s="85"/>
+      <c r="D34" s="85"/>
+      <c r="E34" s="85"/>
+      <c r="F34" s="85"/>
+      <c r="G34" s="85"/>
+      <c r="H34" s="85"/>
+      <c r="I34" s="86"/>
+      <c r="J34" s="81"/>
+      <c r="K34" s="81"/>
+      <c r="L34" s="81"/>
+      <c r="M34" s="81"/>
+      <c r="N34" s="81"/>
+      <c r="O34" s="81"/>
+      <c r="P34" s="86"/>
+      <c r="Q34" s="81"/>
+      <c r="R34" s="81"/>
     </row>
     <row r="35" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A35" s="49"/>
       <c r="B35" s="49"/>
       <c r="C35" s="49"/>
-      <c r="D35" s="68"/>
+      <c r="D35" s="67"/>
       <c r="E35" s="49"/>
       <c r="F35" s="49"/>
       <c r="G35" s="49"/>
@@ -5432,7 +5444,7 @@
       <c r="J35" s="49"/>
       <c r="K35" s="49"/>
       <c r="L35" s="49"/>
-      <c r="M35" s="68"/>
+      <c r="M35" s="67"/>
       <c r="N35" s="49"/>
       <c r="O35" s="49"/>
       <c r="P35" s="49"/>
@@ -5450,8 +5462,8 @@
       <c r="H36" s="49"/>
       <c r="I36" s="49"/>
       <c r="J36" s="49"/>
-      <c r="K36" s="68"/>
-      <c r="L36" s="68"/>
+      <c r="K36" s="67"/>
+      <c r="L36" s="67"/>
       <c r="M36" s="49"/>
       <c r="N36" s="49"/>
       <c r="O36" s="49"/>
@@ -5461,12 +5473,11 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="A22:A24"/>
+    <mergeCell ref="B22:B24"/>
+    <mergeCell ref="C22:H22"/>
+    <mergeCell ref="J22:O22"/>
     <mergeCell ref="Q22:R22"/>
     <mergeCell ref="C23:D23"/>
     <mergeCell ref="E23:F23"/>
@@ -5474,11 +5485,12 @@
     <mergeCell ref="J23:K23"/>
     <mergeCell ref="L23:M23"/>
     <mergeCell ref="N23:O23"/>
-    <mergeCell ref="A7:A9"/>
-    <mergeCell ref="A22:A24"/>
-    <mergeCell ref="B22:B24"/>
-    <mergeCell ref="C22:H22"/>
-    <mergeCell ref="J22:O22"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="I5:J5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5501,385 +5513,385 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="39.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="102" t="s">
+      <c r="A1" s="101" t="s">
         <v>71</v>
       </c>
-      <c r="B1" s="103" t="s">
+      <c r="B1" s="102" t="s">
         <v>72</v>
       </c>
-      <c r="C1" s="103" t="s">
+      <c r="C1" s="102" t="s">
         <v>73</v>
       </c>
-      <c r="D1" s="103" t="s">
+      <c r="D1" s="102" t="s">
         <v>74</v>
       </c>
-      <c r="E1" s="103" t="s">
+      <c r="E1" s="102" t="s">
         <v>75</v>
       </c>
-      <c r="F1" s="103" t="s">
+      <c r="F1" s="102" t="s">
         <v>76</v>
       </c>
-      <c r="G1" s="103" t="s">
+      <c r="G1" s="102" t="s">
         <v>77</v>
       </c>
-      <c r="H1" s="103" t="s">
+      <c r="H1" s="102" t="s">
         <v>78</v>
       </c>
-      <c r="I1" s="104" t="s">
+      <c r="I1" s="103" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="105"/>
-      <c r="B2" s="106"/>
-      <c r="C2" s="107"/>
-      <c r="D2" s="108"/>
-      <c r="E2" s="106"/>
-      <c r="F2" s="106"/>
-      <c r="G2" s="106"/>
-      <c r="H2" s="109"/>
-      <c r="I2" s="110"/>
+      <c r="A2" s="104"/>
+      <c r="B2" s="105"/>
+      <c r="C2" s="106"/>
+      <c r="D2" s="107"/>
+      <c r="E2" s="105"/>
+      <c r="F2" s="105"/>
+      <c r="G2" s="105"/>
+      <c r="H2" s="108"/>
+      <c r="I2" s="109"/>
     </row>
     <row r="3" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="111"/>
-      <c r="B3" s="112"/>
-      <c r="C3" s="113"/>
-      <c r="D3" s="114"/>
-      <c r="E3" s="112"/>
-      <c r="F3" s="112"/>
-      <c r="G3" s="112"/>
-      <c r="H3" s="115"/>
-      <c r="I3" s="116"/>
+      <c r="A3" s="110"/>
+      <c r="B3" s="111"/>
+      <c r="C3" s="112"/>
+      <c r="D3" s="113"/>
+      <c r="E3" s="111"/>
+      <c r="F3" s="111"/>
+      <c r="G3" s="111"/>
+      <c r="H3" s="114"/>
+      <c r="I3" s="115"/>
     </row>
     <row r="4" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="105"/>
-      <c r="B4" s="106"/>
-      <c r="C4" s="107"/>
-      <c r="D4" s="108"/>
-      <c r="E4" s="106"/>
-      <c r="F4" s="106"/>
-      <c r="G4" s="106"/>
-      <c r="H4" s="109"/>
-      <c r="I4" s="110"/>
+      <c r="A4" s="104"/>
+      <c r="B4" s="105"/>
+      <c r="C4" s="106"/>
+      <c r="D4" s="107"/>
+      <c r="E4" s="105"/>
+      <c r="F4" s="105"/>
+      <c r="G4" s="105"/>
+      <c r="H4" s="108"/>
+      <c r="I4" s="109"/>
     </row>
     <row r="5" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="111"/>
-      <c r="B5" s="112"/>
-      <c r="C5" s="113"/>
-      <c r="D5" s="114"/>
-      <c r="E5" s="112"/>
-      <c r="F5" s="112"/>
-      <c r="G5" s="112"/>
-      <c r="H5" s="115"/>
-      <c r="I5" s="116"/>
+      <c r="A5" s="110"/>
+      <c r="B5" s="111"/>
+      <c r="C5" s="112"/>
+      <c r="D5" s="113"/>
+      <c r="E5" s="111"/>
+      <c r="F5" s="111"/>
+      <c r="G5" s="111"/>
+      <c r="H5" s="114"/>
+      <c r="I5" s="115"/>
     </row>
     <row r="6" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="105"/>
-      <c r="B6" s="106"/>
-      <c r="C6" s="107"/>
-      <c r="D6" s="108"/>
-      <c r="E6" s="106"/>
-      <c r="F6" s="106"/>
-      <c r="G6" s="106"/>
-      <c r="H6" s="109"/>
-      <c r="I6" s="117"/>
+      <c r="A6" s="104"/>
+      <c r="B6" s="105"/>
+      <c r="C6" s="106"/>
+      <c r="D6" s="107"/>
+      <c r="E6" s="105"/>
+      <c r="F6" s="105"/>
+      <c r="G6" s="105"/>
+      <c r="H6" s="108"/>
+      <c r="I6" s="116"/>
     </row>
     <row r="7" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="111"/>
-      <c r="B7" s="112"/>
-      <c r="C7" s="113"/>
-      <c r="D7" s="114"/>
-      <c r="E7" s="112"/>
-      <c r="F7" s="112"/>
-      <c r="G7" s="112"/>
-      <c r="H7" s="115"/>
-      <c r="I7" s="118"/>
+      <c r="A7" s="110"/>
+      <c r="B7" s="111"/>
+      <c r="C7" s="112"/>
+      <c r="D7" s="113"/>
+      <c r="E7" s="111"/>
+      <c r="F7" s="111"/>
+      <c r="G7" s="111"/>
+      <c r="H7" s="114"/>
+      <c r="I7" s="117"/>
     </row>
     <row r="8" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="105"/>
-      <c r="B8" s="106"/>
-      <c r="C8" s="107"/>
-      <c r="D8" s="108"/>
-      <c r="E8" s="106"/>
-      <c r="F8" s="106"/>
-      <c r="G8" s="106"/>
-      <c r="H8" s="109"/>
-      <c r="I8" s="117"/>
+      <c r="A8" s="104"/>
+      <c r="B8" s="105"/>
+      <c r="C8" s="106"/>
+      <c r="D8" s="107"/>
+      <c r="E8" s="105"/>
+      <c r="F8" s="105"/>
+      <c r="G8" s="105"/>
+      <c r="H8" s="108"/>
+      <c r="I8" s="116"/>
     </row>
     <row r="9" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="111"/>
-      <c r="B9" s="112"/>
-      <c r="C9" s="113"/>
-      <c r="D9" s="114"/>
-      <c r="E9" s="112"/>
-      <c r="F9" s="112"/>
-      <c r="G9" s="112"/>
-      <c r="H9" s="115"/>
-      <c r="I9" s="119"/>
+      <c r="A9" s="110"/>
+      <c r="B9" s="111"/>
+      <c r="C9" s="112"/>
+      <c r="D9" s="113"/>
+      <c r="E9" s="111"/>
+      <c r="F9" s="111"/>
+      <c r="G9" s="111"/>
+      <c r="H9" s="114"/>
+      <c r="I9" s="118"/>
     </row>
     <row r="10" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="105"/>
-      <c r="B10" s="106"/>
-      <c r="C10" s="107"/>
-      <c r="D10" s="108"/>
-      <c r="E10" s="106"/>
-      <c r="F10" s="106"/>
-      <c r="G10" s="106"/>
-      <c r="H10" s="109"/>
-      <c r="I10" s="120"/>
+      <c r="A10" s="104"/>
+      <c r="B10" s="105"/>
+      <c r="C10" s="106"/>
+      <c r="D10" s="107"/>
+      <c r="E10" s="105"/>
+      <c r="F10" s="105"/>
+      <c r="G10" s="105"/>
+      <c r="H10" s="108"/>
+      <c r="I10" s="119"/>
     </row>
     <row r="11" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="111"/>
-      <c r="B11" s="112"/>
-      <c r="C11" s="113"/>
-      <c r="D11" s="114"/>
-      <c r="E11" s="112"/>
-      <c r="F11" s="112"/>
-      <c r="G11" s="112"/>
-      <c r="H11" s="115"/>
-      <c r="I11" s="121"/>
+      <c r="A11" s="110"/>
+      <c r="B11" s="111"/>
+      <c r="C11" s="112"/>
+      <c r="D11" s="113"/>
+      <c r="E11" s="111"/>
+      <c r="F11" s="111"/>
+      <c r="G11" s="111"/>
+      <c r="H11" s="114"/>
+      <c r="I11" s="120"/>
     </row>
     <row r="12" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="105"/>
-      <c r="B12" s="106"/>
-      <c r="C12" s="107"/>
-      <c r="D12" s="106"/>
-      <c r="E12" s="106"/>
-      <c r="F12" s="106"/>
-      <c r="G12" s="106"/>
-      <c r="H12" s="109"/>
-      <c r="I12" s="120"/>
+      <c r="A12" s="104"/>
+      <c r="B12" s="105"/>
+      <c r="C12" s="106"/>
+      <c r="D12" s="105"/>
+      <c r="E12" s="105"/>
+      <c r="F12" s="105"/>
+      <c r="G12" s="105"/>
+      <c r="H12" s="108"/>
+      <c r="I12" s="119"/>
     </row>
     <row r="13" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="111"/>
-      <c r="B13" s="112"/>
-      <c r="C13" s="113"/>
-      <c r="D13" s="112"/>
-      <c r="E13" s="112"/>
-      <c r="F13" s="112"/>
-      <c r="G13" s="112"/>
-      <c r="H13" s="115"/>
-      <c r="I13" s="121"/>
+      <c r="A13" s="110"/>
+      <c r="B13" s="111"/>
+      <c r="C13" s="112"/>
+      <c r="D13" s="111"/>
+      <c r="E13" s="111"/>
+      <c r="F13" s="111"/>
+      <c r="G13" s="111"/>
+      <c r="H13" s="114"/>
+      <c r="I13" s="120"/>
     </row>
     <row r="14" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="105"/>
-      <c r="B14" s="106"/>
-      <c r="C14" s="107"/>
-      <c r="D14" s="106"/>
-      <c r="E14" s="106"/>
-      <c r="F14" s="106"/>
-      <c r="G14" s="106"/>
-      <c r="H14" s="109"/>
-      <c r="I14" s="120"/>
+      <c r="A14" s="104"/>
+      <c r="B14" s="105"/>
+      <c r="C14" s="106"/>
+      <c r="D14" s="105"/>
+      <c r="E14" s="105"/>
+      <c r="F14" s="105"/>
+      <c r="G14" s="105"/>
+      <c r="H14" s="108"/>
+      <c r="I14" s="119"/>
     </row>
     <row r="15" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="111"/>
-      <c r="B15" s="112"/>
-      <c r="C15" s="113"/>
-      <c r="D15" s="112"/>
-      <c r="E15" s="112"/>
-      <c r="F15" s="112"/>
-      <c r="G15" s="112"/>
-      <c r="H15" s="115"/>
-      <c r="I15" s="121"/>
+      <c r="A15" s="110"/>
+      <c r="B15" s="111"/>
+      <c r="C15" s="112"/>
+      <c r="D15" s="111"/>
+      <c r="E15" s="111"/>
+      <c r="F15" s="111"/>
+      <c r="G15" s="111"/>
+      <c r="H15" s="114"/>
+      <c r="I15" s="120"/>
     </row>
     <row r="16" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="105"/>
-      <c r="B16" s="106"/>
-      <c r="C16" s="107"/>
-      <c r="D16" s="106"/>
-      <c r="E16" s="106"/>
-      <c r="F16" s="106"/>
-      <c r="G16" s="106"/>
-      <c r="H16" s="109"/>
-      <c r="I16" s="120"/>
+      <c r="A16" s="104"/>
+      <c r="B16" s="105"/>
+      <c r="C16" s="106"/>
+      <c r="D16" s="105"/>
+      <c r="E16" s="105"/>
+      <c r="F16" s="105"/>
+      <c r="G16" s="105"/>
+      <c r="H16" s="108"/>
+      <c r="I16" s="119"/>
     </row>
     <row r="17" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="111"/>
-      <c r="B17" s="112"/>
-      <c r="C17" s="113"/>
-      <c r="D17" s="114"/>
-      <c r="E17" s="112"/>
-      <c r="F17" s="112"/>
-      <c r="G17" s="112"/>
-      <c r="H17" s="115"/>
-      <c r="I17" s="121"/>
+      <c r="A17" s="110"/>
+      <c r="B17" s="111"/>
+      <c r="C17" s="112"/>
+      <c r="D17" s="113"/>
+      <c r="E17" s="111"/>
+      <c r="F17" s="111"/>
+      <c r="G17" s="111"/>
+      <c r="H17" s="114"/>
+      <c r="I17" s="120"/>
     </row>
     <row r="18" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="105"/>
-      <c r="B18" s="106"/>
-      <c r="C18" s="106"/>
-      <c r="D18" s="106"/>
-      <c r="E18" s="106"/>
-      <c r="F18" s="106"/>
-      <c r="G18" s="106"/>
-      <c r="H18" s="109"/>
-      <c r="I18" s="110"/>
+      <c r="A18" s="104"/>
+      <c r="B18" s="105"/>
+      <c r="C18" s="105"/>
+      <c r="D18" s="105"/>
+      <c r="E18" s="105"/>
+      <c r="F18" s="105"/>
+      <c r="G18" s="105"/>
+      <c r="H18" s="108"/>
+      <c r="I18" s="109"/>
     </row>
     <row r="19" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="111"/>
-      <c r="B19" s="112"/>
-      <c r="C19" s="113"/>
-      <c r="D19" s="112"/>
-      <c r="E19" s="112"/>
-      <c r="F19" s="112"/>
-      <c r="G19" s="112"/>
-      <c r="H19" s="115"/>
-      <c r="I19" s="121"/>
+      <c r="A19" s="110"/>
+      <c r="B19" s="111"/>
+      <c r="C19" s="112"/>
+      <c r="D19" s="111"/>
+      <c r="E19" s="111"/>
+      <c r="F19" s="111"/>
+      <c r="G19" s="111"/>
+      <c r="H19" s="114"/>
+      <c r="I19" s="120"/>
     </row>
     <row r="20" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="105"/>
-      <c r="B20" s="106"/>
-      <c r="C20" s="107"/>
-      <c r="D20" s="106"/>
-      <c r="E20" s="106"/>
-      <c r="F20" s="106"/>
-      <c r="G20" s="106"/>
-      <c r="H20" s="109"/>
-      <c r="I20" s="120"/>
+      <c r="A20" s="104"/>
+      <c r="B20" s="105"/>
+      <c r="C20" s="106"/>
+      <c r="D20" s="105"/>
+      <c r="E20" s="105"/>
+      <c r="F20" s="105"/>
+      <c r="G20" s="105"/>
+      <c r="H20" s="108"/>
+      <c r="I20" s="119"/>
     </row>
     <row r="21" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="111"/>
-      <c r="B21" s="112"/>
-      <c r="C21" s="113"/>
-      <c r="D21" s="112"/>
-      <c r="E21" s="112"/>
-      <c r="F21" s="112"/>
-      <c r="G21" s="112"/>
-      <c r="H21" s="115"/>
-      <c r="I21" s="121"/>
+      <c r="A21" s="110"/>
+      <c r="B21" s="111"/>
+      <c r="C21" s="112"/>
+      <c r="D21" s="111"/>
+      <c r="E21" s="111"/>
+      <c r="F21" s="111"/>
+      <c r="G21" s="111"/>
+      <c r="H21" s="114"/>
+      <c r="I21" s="120"/>
     </row>
     <row r="22" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="105"/>
-      <c r="B22" s="106"/>
-      <c r="C22" s="107"/>
-      <c r="D22" s="106"/>
-      <c r="E22" s="106"/>
-      <c r="F22" s="106"/>
-      <c r="G22" s="106"/>
-      <c r="H22" s="109"/>
-      <c r="I22" s="117"/>
+      <c r="A22" s="104"/>
+      <c r="B22" s="105"/>
+      <c r="C22" s="106"/>
+      <c r="D22" s="105"/>
+      <c r="E22" s="105"/>
+      <c r="F22" s="105"/>
+      <c r="G22" s="105"/>
+      <c r="H22" s="108"/>
+      <c r="I22" s="116"/>
     </row>
     <row r="23" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="111"/>
-      <c r="B23" s="112"/>
-      <c r="C23" s="113"/>
-      <c r="D23" s="112"/>
-      <c r="E23" s="112"/>
-      <c r="F23" s="112"/>
-      <c r="G23" s="112"/>
-      <c r="H23" s="115"/>
-      <c r="I23" s="118"/>
+      <c r="A23" s="110"/>
+      <c r="B23" s="111"/>
+      <c r="C23" s="112"/>
+      <c r="D23" s="111"/>
+      <c r="E23" s="111"/>
+      <c r="F23" s="111"/>
+      <c r="G23" s="111"/>
+      <c r="H23" s="114"/>
+      <c r="I23" s="117"/>
     </row>
     <row r="24" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="105"/>
-      <c r="B24" s="106"/>
-      <c r="C24" s="107"/>
-      <c r="D24" s="106"/>
-      <c r="E24" s="106"/>
-      <c r="F24" s="106"/>
-      <c r="G24" s="106"/>
-      <c r="H24" s="109"/>
-      <c r="I24" s="117"/>
+      <c r="A24" s="104"/>
+      <c r="B24" s="105"/>
+      <c r="C24" s="106"/>
+      <c r="D24" s="105"/>
+      <c r="E24" s="105"/>
+      <c r="F24" s="105"/>
+      <c r="G24" s="105"/>
+      <c r="H24" s="108"/>
+      <c r="I24" s="116"/>
     </row>
     <row r="25" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="111"/>
-      <c r="B25" s="112"/>
-      <c r="C25" s="113"/>
-      <c r="D25" s="112"/>
-      <c r="E25" s="112"/>
-      <c r="F25" s="112"/>
-      <c r="G25" s="112"/>
-      <c r="H25" s="115"/>
-      <c r="I25" s="118"/>
+      <c r="A25" s="110"/>
+      <c r="B25" s="111"/>
+      <c r="C25" s="112"/>
+      <c r="D25" s="111"/>
+      <c r="E25" s="111"/>
+      <c r="F25" s="111"/>
+      <c r="G25" s="111"/>
+      <c r="H25" s="114"/>
+      <c r="I25" s="117"/>
     </row>
     <row r="26" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="105"/>
-      <c r="B26" s="106"/>
-      <c r="C26" s="107"/>
-      <c r="D26" s="106"/>
-      <c r="E26" s="106"/>
-      <c r="F26" s="106"/>
-      <c r="G26" s="106"/>
-      <c r="H26" s="109"/>
-      <c r="I26" s="117"/>
+      <c r="A26" s="104"/>
+      <c r="B26" s="105"/>
+      <c r="C26" s="106"/>
+      <c r="D26" s="105"/>
+      <c r="E26" s="105"/>
+      <c r="F26" s="105"/>
+      <c r="G26" s="105"/>
+      <c r="H26" s="108"/>
+      <c r="I26" s="116"/>
     </row>
     <row r="27" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="111"/>
-      <c r="B27" s="112"/>
-      <c r="C27" s="113"/>
-      <c r="D27" s="112"/>
-      <c r="E27" s="112"/>
-      <c r="F27" s="112"/>
-      <c r="G27" s="112"/>
-      <c r="H27" s="115"/>
-      <c r="I27" s="118"/>
+      <c r="A27" s="110"/>
+      <c r="B27" s="111"/>
+      <c r="C27" s="112"/>
+      <c r="D27" s="111"/>
+      <c r="E27" s="111"/>
+      <c r="F27" s="111"/>
+      <c r="G27" s="111"/>
+      <c r="H27" s="114"/>
+      <c r="I27" s="117"/>
     </row>
     <row r="28" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="105"/>
-      <c r="B28" s="106"/>
-      <c r="C28" s="107"/>
-      <c r="D28" s="106"/>
-      <c r="E28" s="106"/>
-      <c r="F28" s="106"/>
-      <c r="G28" s="106"/>
-      <c r="H28" s="109"/>
-      <c r="I28" s="117"/>
+      <c r="A28" s="104"/>
+      <c r="B28" s="105"/>
+      <c r="C28" s="106"/>
+      <c r="D28" s="105"/>
+      <c r="E28" s="105"/>
+      <c r="F28" s="105"/>
+      <c r="G28" s="105"/>
+      <c r="H28" s="108"/>
+      <c r="I28" s="116"/>
     </row>
     <row r="29" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="111"/>
-      <c r="B29" s="112"/>
-      <c r="C29" s="113"/>
-      <c r="D29" s="112"/>
-      <c r="E29" s="112"/>
-      <c r="F29" s="112"/>
-      <c r="G29" s="112"/>
-      <c r="H29" s="115"/>
-      <c r="I29" s="118"/>
+      <c r="A29" s="110"/>
+      <c r="B29" s="111"/>
+      <c r="C29" s="112"/>
+      <c r="D29" s="111"/>
+      <c r="E29" s="111"/>
+      <c r="F29" s="111"/>
+      <c r="G29" s="111"/>
+      <c r="H29" s="114"/>
+      <c r="I29" s="117"/>
     </row>
     <row r="30" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="105"/>
-      <c r="B30" s="106"/>
-      <c r="C30" s="107"/>
-      <c r="D30" s="106"/>
-      <c r="E30" s="106"/>
-      <c r="F30" s="106"/>
-      <c r="G30" s="106"/>
-      <c r="H30" s="109"/>
-      <c r="I30" s="117"/>
+      <c r="A30" s="104"/>
+      <c r="B30" s="105"/>
+      <c r="C30" s="106"/>
+      <c r="D30" s="105"/>
+      <c r="E30" s="105"/>
+      <c r="F30" s="105"/>
+      <c r="G30" s="105"/>
+      <c r="H30" s="108"/>
+      <c r="I30" s="116"/>
     </row>
     <row r="31" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="111"/>
-      <c r="B31" s="112"/>
-      <c r="C31" s="113"/>
-      <c r="D31" s="112"/>
-      <c r="E31" s="112"/>
-      <c r="F31" s="112"/>
-      <c r="G31" s="112"/>
-      <c r="H31" s="115"/>
-      <c r="I31" s="118"/>
+      <c r="A31" s="110"/>
+      <c r="B31" s="111"/>
+      <c r="C31" s="112"/>
+      <c r="D31" s="111"/>
+      <c r="E31" s="111"/>
+      <c r="F31" s="111"/>
+      <c r="G31" s="111"/>
+      <c r="H31" s="114"/>
+      <c r="I31" s="117"/>
     </row>
     <row r="32" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="105"/>
-      <c r="B32" s="106"/>
-      <c r="C32" s="107"/>
-      <c r="D32" s="106"/>
-      <c r="E32" s="106"/>
-      <c r="F32" s="106"/>
-      <c r="G32" s="106"/>
-      <c r="H32" s="122"/>
-      <c r="I32" s="117"/>
+      <c r="A32" s="104"/>
+      <c r="B32" s="105"/>
+      <c r="C32" s="106"/>
+      <c r="D32" s="105"/>
+      <c r="E32" s="105"/>
+      <c r="F32" s="105"/>
+      <c r="G32" s="105"/>
+      <c r="H32" s="121"/>
+      <c r="I32" s="116"/>
     </row>
     <row r="33" spans="1:9" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="123"/>
-      <c r="B33" s="124"/>
-      <c r="C33" s="124"/>
-      <c r="D33" s="124"/>
-      <c r="E33" s="124"/>
-      <c r="F33" s="124"/>
-      <c r="G33" s="124"/>
-      <c r="H33" s="124"/>
-      <c r="I33" s="119"/>
+      <c r="A33" s="122"/>
+      <c r="B33" s="123"/>
+      <c r="C33" s="123"/>
+      <c r="D33" s="123"/>
+      <c r="E33" s="123"/>
+      <c r="F33" s="123"/>
+      <c r="G33" s="123"/>
+      <c r="H33" s="123"/>
+      <c r="I33" s="118"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Fixed Some Bugs and Added QoL
</commit_message>
<xml_diff>
--- a/backend/utils/template2.xlsx
+++ b/backend/utils/template2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\My Stuff\Github\IPCR_GENERATOR-Thesis\backend\utils\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D21EDC5-F16B-40D5-B394-548954DB5318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80D36098-E259-4CF9-9265-22E5E32002CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1st Quarter" sheetId="1" r:id="rId1"/>
@@ -1130,7 +1130,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="162">
+  <cellXfs count="161">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1385,15 +1385,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="16" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1499,86 +1490,14 @@
     <xf numFmtId="0" fontId="34" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="13" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="13" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="14" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="14" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1590,6 +1509,15 @@
     <xf numFmtId="0" fontId="30" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1599,10 +1527,79 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="14" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="14" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="16" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1886,16 +1883,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="102.75" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="152" t="s">
+      <c r="A1" s="136" t="s">
         <v>80</v>
       </c>
-      <c r="B1" s="153"/>
-      <c r="C1" s="153"/>
-      <c r="D1" s="153"/>
-      <c r="E1" s="153"/>
-      <c r="F1" s="153"/>
-      <c r="G1" s="153"/>
-      <c r="H1" s="153"/>
+      <c r="B1" s="126"/>
+      <c r="C1" s="126"/>
+      <c r="D1" s="126"/>
+      <c r="E1" s="126"/>
+      <c r="F1" s="126"/>
+      <c r="G1" s="126"/>
+      <c r="H1" s="126"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
     </row>
@@ -2442,16 +2439,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="102.75" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="152" t="s">
+      <c r="A1" s="136" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="153"/>
-      <c r="C1" s="153"/>
-      <c r="D1" s="153"/>
-      <c r="E1" s="153"/>
-      <c r="F1" s="153"/>
-      <c r="G1" s="153"/>
-      <c r="H1" s="153"/>
+      <c r="B1" s="126"/>
+      <c r="C1" s="126"/>
+      <c r="D1" s="126"/>
+      <c r="E1" s="126"/>
+      <c r="F1" s="126"/>
+      <c r="G1" s="126"/>
+      <c r="H1" s="126"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
     </row>
@@ -3002,16 +2999,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="102.75" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="152" t="s">
+      <c r="A1" s="136" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="153"/>
-      <c r="C1" s="153"/>
-      <c r="D1" s="153"/>
-      <c r="E1" s="153"/>
-      <c r="F1" s="153"/>
-      <c r="G1" s="153"/>
-      <c r="H1" s="153"/>
+      <c r="B1" s="126"/>
+      <c r="C1" s="126"/>
+      <c r="D1" s="126"/>
+      <c r="E1" s="126"/>
+      <c r="F1" s="126"/>
+      <c r="G1" s="126"/>
+      <c r="H1" s="126"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
     </row>
@@ -3562,16 +3559,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="102.75" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="152" t="s">
+      <c r="A1" s="136" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="153"/>
-      <c r="C1" s="153"/>
-      <c r="D1" s="153"/>
-      <c r="E1" s="153"/>
-      <c r="F1" s="153"/>
-      <c r="G1" s="153"/>
-      <c r="H1" s="153"/>
+      <c r="B1" s="126"/>
+      <c r="C1" s="126"/>
+      <c r="D1" s="126"/>
+      <c r="E1" s="126"/>
+      <c r="F1" s="126"/>
+      <c r="G1" s="126"/>
+      <c r="H1" s="126"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
     </row>
@@ -4133,20 +4130,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:30" ht="29.25" thickBot="1" x14ac:dyDescent="0.85">
-      <c r="A1" s="126" t="s">
+      <c r="A1" s="130" t="s">
         <v>46</v>
       </c>
-      <c r="B1" s="127"/>
-      <c r="C1" s="127"/>
-      <c r="D1" s="127"/>
-      <c r="E1" s="127"/>
-      <c r="F1" s="127"/>
-      <c r="G1" s="127"/>
-      <c r="H1" s="127"/>
-      <c r="I1" s="127"/>
-      <c r="J1" s="127"/>
-      <c r="K1" s="127"/>
-      <c r="L1" s="128"/>
+      <c r="B1" s="131"/>
+      <c r="C1" s="131"/>
+      <c r="D1" s="131"/>
+      <c r="E1" s="131"/>
+      <c r="F1" s="131"/>
+      <c r="G1" s="131"/>
+      <c r="H1" s="131"/>
+      <c r="I1" s="131"/>
+      <c r="J1" s="131"/>
+      <c r="K1" s="131"/>
+      <c r="L1" s="132"/>
       <c r="M1" t="s">
         <v>47</v>
       </c>
@@ -4155,13 +4152,13 @@
       <c r="A2" s="87" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="88"/>
-      <c r="C2" s="157" t="s">
+      <c r="B2" s="125"/>
+      <c r="C2" s="133" t="s">
         <v>49</v>
       </c>
-      <c r="D2" s="158"/>
-      <c r="E2" s="159"/>
-      <c r="F2" s="89"/>
+      <c r="D2" s="134"/>
+      <c r="E2" s="135"/>
+      <c r="F2" s="125"/>
       <c r="G2" s="49"/>
       <c r="H2" s="49"/>
       <c r="I2" s="49"/>
@@ -4173,13 +4170,13 @@
       <c r="A3" s="87" t="s">
         <v>50</v>
       </c>
-      <c r="B3" s="90"/>
-      <c r="C3" s="157" t="s">
+      <c r="B3" s="124"/>
+      <c r="C3" s="133" t="s">
         <v>51</v>
       </c>
-      <c r="D3" s="158"/>
-      <c r="E3" s="159"/>
-      <c r="F3" s="88"/>
+      <c r="D3" s="134"/>
+      <c r="E3" s="135"/>
+      <c r="F3" s="160"/>
       <c r="G3" s="49"/>
       <c r="H3" s="49"/>
       <c r="I3" s="49"/>
@@ -4191,13 +4188,13 @@
       <c r="A4" s="87" t="s">
         <v>52</v>
       </c>
-      <c r="B4" s="90"/>
-      <c r="C4" s="157" t="s">
+      <c r="B4" s="124"/>
+      <c r="C4" s="133" t="s">
         <v>53</v>
       </c>
-      <c r="D4" s="158"/>
-      <c r="E4" s="159"/>
-      <c r="F4" s="88"/>
+      <c r="D4" s="134"/>
+      <c r="E4" s="135"/>
+      <c r="F4" s="160"/>
       <c r="G4" s="49"/>
       <c r="H4" s="49"/>
       <c r="I4" s="49"/>
@@ -4206,133 +4203,133 @@
       <c r="L4" s="49"/>
     </row>
     <row r="5" spans="1:30" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="91"/>
-      <c r="B5" s="91"/>
-      <c r="C5" s="91"/>
-      <c r="D5" s="91"/>
+      <c r="A5" s="88"/>
+      <c r="B5" s="88"/>
+      <c r="C5" s="88"/>
+      <c r="D5" s="88"/>
       <c r="E5" s="58"/>
       <c r="F5" s="58"/>
-      <c r="G5" s="91"/>
-      <c r="H5" s="91"/>
-      <c r="I5" s="91"/>
-      <c r="J5" s="91"/>
+      <c r="G5" s="88"/>
+      <c r="H5" s="88"/>
+      <c r="I5" s="88"/>
+      <c r="J5" s="88"/>
       <c r="K5" s="49"/>
       <c r="L5" s="49"/>
     </row>
     <row r="6" spans="1:30" ht="41.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="92" t="s">
+      <c r="A6" s="89" t="s">
         <v>54</v>
       </c>
-      <c r="B6" s="93"/>
-      <c r="C6" s="93"/>
-      <c r="D6" s="93"/>
-      <c r="E6" s="93"/>
-      <c r="F6" s="93"/>
-      <c r="G6" s="93"/>
-      <c r="H6" s="93"/>
-      <c r="I6" s="93"/>
-      <c r="J6" s="93"/>
+      <c r="B6" s="90"/>
+      <c r="C6" s="90"/>
+      <c r="D6" s="90"/>
+      <c r="E6" s="90"/>
+      <c r="F6" s="90"/>
+      <c r="G6" s="90"/>
+      <c r="H6" s="90"/>
+      <c r="I6" s="90"/>
+      <c r="J6" s="90"/>
       <c r="K6" s="49"/>
       <c r="L6" s="49"/>
-      <c r="U6" s="153"/>
-      <c r="V6" s="153"/>
+      <c r="U6" s="126"/>
+      <c r="V6" s="126"/>
     </row>
     <row r="7" spans="1:30" ht="67.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="94" t="s">
+      <c r="A7" s="91" t="s">
         <v>55</v>
       </c>
-      <c r="B7" s="124"/>
-      <c r="C7" s="124"/>
-      <c r="D7" s="124"/>
-      <c r="E7" s="124"/>
-      <c r="F7" s="124"/>
-      <c r="G7" s="124"/>
-      <c r="H7" s="124"/>
-      <c r="I7" s="124"/>
-      <c r="J7" s="124"/>
+      <c r="B7" s="121"/>
+      <c r="C7" s="121"/>
+      <c r="D7" s="121"/>
+      <c r="E7" s="121"/>
+      <c r="F7" s="121"/>
+      <c r="G7" s="121"/>
+      <c r="H7" s="121"/>
+      <c r="I7" s="121"/>
+      <c r="J7" s="121"/>
       <c r="K7" s="49"/>
       <c r="L7" s="49"/>
-      <c r="U7" s="153"/>
-      <c r="V7" s="153"/>
+      <c r="U7" s="126"/>
+      <c r="V7" s="126"/>
     </row>
     <row r="8" spans="1:30" ht="49.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="A8" s="94" t="s">
+      <c r="A8" s="91" t="s">
         <v>56</v>
       </c>
-      <c r="B8" s="124"/>
-      <c r="C8" s="125"/>
-      <c r="D8" s="124"/>
-      <c r="E8" s="124"/>
-      <c r="F8" s="125"/>
-      <c r="G8" s="124"/>
-      <c r="H8" s="125"/>
-      <c r="I8" s="124"/>
-      <c r="J8" s="124"/>
-      <c r="K8" s="95"/>
+      <c r="B8" s="121"/>
+      <c r="C8" s="122"/>
+      <c r="D8" s="121"/>
+      <c r="E8" s="121"/>
+      <c r="F8" s="122"/>
+      <c r="G8" s="121"/>
+      <c r="H8" s="122"/>
+      <c r="I8" s="121"/>
+      <c r="J8" s="121"/>
+      <c r="K8" s="92"/>
       <c r="L8" s="49"/>
     </row>
     <row r="9" spans="1:30" ht="41.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="A9" s="94" t="s">
+      <c r="A9" s="91" t="s">
         <v>57</v>
       </c>
-      <c r="B9" s="124"/>
-      <c r="C9" s="124"/>
-      <c r="D9" s="125"/>
-      <c r="E9" s="124"/>
-      <c r="F9" s="124"/>
-      <c r="G9" s="124"/>
-      <c r="H9" s="124"/>
-      <c r="I9" s="124"/>
-      <c r="J9" s="124"/>
-      <c r="K9" s="95"/>
+      <c r="B9" s="121"/>
+      <c r="C9" s="121"/>
+      <c r="D9" s="122"/>
+      <c r="E9" s="121"/>
+      <c r="F9" s="121"/>
+      <c r="G9" s="121"/>
+      <c r="H9" s="121"/>
+      <c r="I9" s="121"/>
+      <c r="J9" s="121"/>
+      <c r="K9" s="92"/>
       <c r="L9" s="49"/>
     </row>
     <row r="10" spans="1:30" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="A10" s="94" t="s">
+      <c r="A10" s="91" t="s">
         <v>58</v>
       </c>
-      <c r="B10" s="125"/>
-      <c r="C10" s="124"/>
-      <c r="D10" s="125"/>
-      <c r="E10" s="125"/>
-      <c r="F10" s="124"/>
-      <c r="G10" s="124"/>
-      <c r="H10" s="124"/>
-      <c r="I10" s="124"/>
-      <c r="J10" s="125"/>
-      <c r="K10" s="95"/>
+      <c r="B10" s="122"/>
+      <c r="C10" s="121"/>
+      <c r="D10" s="122"/>
+      <c r="E10" s="122"/>
+      <c r="F10" s="121"/>
+      <c r="G10" s="121"/>
+      <c r="H10" s="121"/>
+      <c r="I10" s="121"/>
+      <c r="J10" s="122"/>
+      <c r="K10" s="92"/>
       <c r="L10" s="49"/>
     </row>
     <row r="11" spans="1:30" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="A11" s="94" t="s">
+      <c r="A11" s="91" t="s">
         <v>59</v>
       </c>
-      <c r="B11" s="124"/>
-      <c r="C11" s="124"/>
-      <c r="D11" s="124"/>
-      <c r="E11" s="124"/>
-      <c r="F11" s="124"/>
-      <c r="G11" s="124"/>
-      <c r="H11" s="124"/>
-      <c r="I11" s="124"/>
-      <c r="J11" s="124"/>
-      <c r="K11" s="95"/>
+      <c r="B11" s="121"/>
+      <c r="C11" s="121"/>
+      <c r="D11" s="121"/>
+      <c r="E11" s="121"/>
+      <c r="F11" s="121"/>
+      <c r="G11" s="121"/>
+      <c r="H11" s="121"/>
+      <c r="I11" s="121"/>
+      <c r="J11" s="121"/>
+      <c r="K11" s="92"/>
       <c r="L11" s="49"/>
     </row>
     <row r="12" spans="1:30" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="A12" s="94" t="s">
+      <c r="A12" s="91" t="s">
         <v>60</v>
       </c>
-      <c r="B12" s="124"/>
-      <c r="C12" s="124"/>
-      <c r="D12" s="124"/>
-      <c r="E12" s="124"/>
-      <c r="F12" s="124"/>
-      <c r="G12" s="124"/>
-      <c r="H12" s="124"/>
-      <c r="I12" s="124"/>
-      <c r="J12" s="124"/>
-      <c r="K12" s="95"/>
+      <c r="B12" s="121"/>
+      <c r="C12" s="121"/>
+      <c r="D12" s="121"/>
+      <c r="E12" s="121"/>
+      <c r="F12" s="121"/>
+      <c r="G12" s="121"/>
+      <c r="H12" s="121"/>
+      <c r="I12" s="121"/>
+      <c r="J12" s="121"/>
+      <c r="K12" s="92"/>
       <c r="L12" s="49"/>
     </row>
     <row r="13" spans="1:30" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
@@ -4377,11 +4374,11 @@
       <c r="A15" s="87" t="s">
         <v>61</v>
       </c>
-      <c r="B15" s="154" t="s">
+      <c r="B15" s="127" t="s">
         <v>62</v>
       </c>
-      <c r="C15" s="155"/>
-      <c r="D15" s="156"/>
+      <c r="C15" s="128"/>
+      <c r="D15" s="129"/>
       <c r="E15" s="49"/>
       <c r="F15" s="49"/>
       <c r="G15" s="49"/>
@@ -4397,14 +4394,14 @@
       <c r="AD15" s="49"/>
     </row>
     <row r="16" spans="1:30" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="96"/>
-      <c r="B16" s="97" t="s">
+      <c r="A16" s="93"/>
+      <c r="B16" s="94" t="s">
         <v>63</v>
       </c>
-      <c r="C16" s="97" t="s">
+      <c r="C16" s="94" t="s">
         <v>64</v>
       </c>
-      <c r="D16" s="97" t="s">
+      <c r="D16" s="94" t="s">
         <v>65</v>
       </c>
       <c r="E16" s="49"/>
@@ -4422,10 +4419,10 @@
       <c r="AD16" s="49"/>
     </row>
     <row r="17" spans="1:30" ht="24" thickBot="1" x14ac:dyDescent="0.7">
-      <c r="A17" s="96"/>
-      <c r="B17" s="98"/>
-      <c r="C17" s="98"/>
-      <c r="D17" s="98"/>
+      <c r="A17" s="93"/>
+      <c r="B17" s="95"/>
+      <c r="C17" s="95"/>
+      <c r="D17" s="95"/>
       <c r="E17" s="49"/>
       <c r="F17" s="49"/>
       <c r="G17" s="49"/>
@@ -4479,7 +4476,7 @@
       <c r="AD19" s="49"/>
     </row>
     <row r="20" spans="1:30" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A20" s="99" t="s">
+      <c r="A20" s="96" t="s">
         <v>66</v>
       </c>
       <c r="B20" s="49"/>
@@ -4503,7 +4500,7 @@
       <c r="A21" s="66" t="s">
         <v>67</v>
       </c>
-      <c r="B21" s="100"/>
+      <c r="B21" s="97"/>
       <c r="C21" s="49"/>
       <c r="D21" s="49"/>
       <c r="E21" s="49"/>
@@ -4524,7 +4521,7 @@
       <c r="A22" s="66" t="s">
         <v>68</v>
       </c>
-      <c r="B22" s="100"/>
+      <c r="B22" s="97"/>
       <c r="C22" s="49"/>
       <c r="D22" s="49"/>
       <c r="E22" s="49"/>
@@ -4545,7 +4542,7 @@
       <c r="A23" s="66" t="s">
         <v>69</v>
       </c>
-      <c r="B23" s="100"/>
+      <c r="B23" s="97"/>
       <c r="C23" s="49"/>
       <c r="D23" s="49"/>
       <c r="E23" s="49"/>
@@ -4566,7 +4563,7 @@
       <c r="A24" s="66" t="s">
         <v>70</v>
       </c>
-      <c r="B24" s="100"/>
+      <c r="B24" s="97"/>
       <c r="C24" s="49"/>
       <c r="D24" s="49"/>
       <c r="E24" s="49"/>
@@ -4620,20 +4617,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="29.25" thickBot="1" x14ac:dyDescent="0.85">
-      <c r="A1" s="126" t="s">
+      <c r="A1" s="130" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="127"/>
-      <c r="C1" s="127"/>
-      <c r="D1" s="127"/>
-      <c r="E1" s="127"/>
-      <c r="F1" s="127"/>
-      <c r="G1" s="127"/>
-      <c r="H1" s="127"/>
-      <c r="I1" s="127"/>
-      <c r="J1" s="127"/>
-      <c r="K1" s="127"/>
-      <c r="L1" s="128"/>
+      <c r="B1" s="131"/>
+      <c r="C1" s="131"/>
+      <c r="D1" s="131"/>
+      <c r="E1" s="131"/>
+      <c r="F1" s="131"/>
+      <c r="G1" s="131"/>
+      <c r="H1" s="131"/>
+      <c r="I1" s="131"/>
+      <c r="J1" s="131"/>
+      <c r="K1" s="131"/>
+      <c r="L1" s="132"/>
       <c r="M1" s="49"/>
       <c r="N1" s="49"/>
       <c r="O1" s="49"/>
@@ -4642,10 +4639,10 @@
       <c r="R1" s="49"/>
     </row>
     <row r="2" spans="1:18" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.7">
-      <c r="A2" s="129" t="s">
+      <c r="A2" s="137" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="130"/>
+      <c r="B2" s="138"/>
       <c r="C2" s="50"/>
       <c r="D2" s="49"/>
       <c r="E2" s="49"/>
@@ -4710,22 +4707,22 @@
       <c r="B5" s="54" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="131" t="s">
+      <c r="C5" s="139" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="132"/>
-      <c r="E5" s="133" t="s">
+      <c r="D5" s="140"/>
+      <c r="E5" s="141" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="134"/>
-      <c r="G5" s="135" t="s">
+      <c r="F5" s="142"/>
+      <c r="G5" s="143" t="s">
         <v>18</v>
       </c>
-      <c r="H5" s="136"/>
-      <c r="I5" s="137" t="s">
+      <c r="H5" s="144"/>
+      <c r="I5" s="145" t="s">
         <v>19</v>
       </c>
-      <c r="J5" s="138"/>
+      <c r="J5" s="146"/>
       <c r="K5" s="54" t="s">
         <v>20</v>
       </c>
@@ -4776,22 +4773,22 @@
       <c r="R6" s="55"/>
     </row>
     <row r="7" spans="1:18" ht="50.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="145" t="s">
+      <c r="A7" s="153" t="s">
         <v>24</v>
       </c>
       <c r="B7" s="59" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="160"/>
-      <c r="D7" s="160"/>
-      <c r="E7" s="160"/>
-      <c r="F7" s="161"/>
-      <c r="G7" s="160"/>
-      <c r="H7" s="161"/>
-      <c r="I7" s="160"/>
-      <c r="J7" s="161"/>
-      <c r="K7" s="160"/>
-      <c r="L7" s="160"/>
+      <c r="C7" s="90"/>
+      <c r="D7" s="90"/>
+      <c r="E7" s="90"/>
+      <c r="F7" s="123"/>
+      <c r="G7" s="90"/>
+      <c r="H7" s="123"/>
+      <c r="I7" s="90"/>
+      <c r="J7" s="123"/>
+      <c r="K7" s="90"/>
+      <c r="L7" s="90"/>
       <c r="M7" s="49"/>
       <c r="N7" s="49"/>
       <c r="O7" s="49"/>
@@ -4800,20 +4797,20 @@
       <c r="R7" s="49"/>
     </row>
     <row r="8" spans="1:18" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A8" s="146"/>
+      <c r="A8" s="154"/>
       <c r="B8" s="60" t="s">
         <v>26</v>
       </c>
-      <c r="C8" s="160"/>
-      <c r="D8" s="160"/>
-      <c r="E8" s="160"/>
-      <c r="F8" s="161"/>
-      <c r="G8" s="160"/>
-      <c r="H8" s="161"/>
-      <c r="I8" s="160"/>
-      <c r="J8" s="161"/>
-      <c r="K8" s="160"/>
-      <c r="L8" s="160"/>
+      <c r="C8" s="90"/>
+      <c r="D8" s="90"/>
+      <c r="E8" s="90"/>
+      <c r="F8" s="123"/>
+      <c r="G8" s="90"/>
+      <c r="H8" s="123"/>
+      <c r="I8" s="90"/>
+      <c r="J8" s="123"/>
+      <c r="K8" s="90"/>
+      <c r="L8" s="90"/>
       <c r="M8" s="49"/>
       <c r="N8" s="49"/>
       <c r="O8" s="49"/>
@@ -4822,20 +4819,20 @@
       <c r="R8" s="49"/>
     </row>
     <row r="9" spans="1:18" ht="39.75" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A9" s="147"/>
+      <c r="A9" s="155"/>
       <c r="B9" s="60" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="160"/>
-      <c r="D9" s="160"/>
-      <c r="E9" s="160"/>
-      <c r="F9" s="161"/>
-      <c r="G9" s="160"/>
-      <c r="H9" s="161"/>
-      <c r="I9" s="160"/>
-      <c r="J9" s="161"/>
-      <c r="K9" s="160"/>
-      <c r="L9" s="160"/>
+      <c r="C9" s="90"/>
+      <c r="D9" s="90"/>
+      <c r="E9" s="90"/>
+      <c r="F9" s="123"/>
+      <c r="G9" s="90"/>
+      <c r="H9" s="123"/>
+      <c r="I9" s="90"/>
+      <c r="J9" s="123"/>
+      <c r="K9" s="90"/>
+      <c r="L9" s="90"/>
       <c r="M9" s="49"/>
       <c r="N9" s="49"/>
       <c r="O9" s="49"/>
@@ -5122,63 +5119,63 @@
       <c r="R21" s="52"/>
     </row>
     <row r="22" spans="1:18" ht="20.25" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A22" s="148" t="s">
+      <c r="A22" s="156" t="s">
         <v>37</v>
       </c>
-      <c r="B22" s="148" t="s">
+      <c r="B22" s="156" t="s">
         <v>38</v>
       </c>
-      <c r="C22" s="139" t="s">
+      <c r="C22" s="147" t="s">
         <v>39</v>
       </c>
-      <c r="D22" s="151"/>
-      <c r="E22" s="151"/>
-      <c r="F22" s="151"/>
-      <c r="G22" s="151"/>
-      <c r="H22" s="140"/>
+      <c r="D22" s="159"/>
+      <c r="E22" s="159"/>
+      <c r="F22" s="159"/>
+      <c r="G22" s="159"/>
+      <c r="H22" s="148"/>
       <c r="I22" s="57"/>
-      <c r="J22" s="139" t="s">
+      <c r="J22" s="147" t="s">
         <v>40</v>
       </c>
-      <c r="K22" s="151"/>
-      <c r="L22" s="151"/>
-      <c r="M22" s="151"/>
-      <c r="N22" s="151"/>
-      <c r="O22" s="140"/>
+      <c r="K22" s="159"/>
+      <c r="L22" s="159"/>
+      <c r="M22" s="159"/>
+      <c r="N22" s="159"/>
+      <c r="O22" s="148"/>
       <c r="P22" s="57"/>
-      <c r="Q22" s="139">
+      <c r="Q22" s="147">
         <v>2025</v>
       </c>
-      <c r="R22" s="140"/>
+      <c r="R22" s="148"/>
     </row>
     <row r="23" spans="1:18" ht="39.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="149"/>
-      <c r="B23" s="149"/>
-      <c r="C23" s="141" t="s">
+      <c r="A23" s="157"/>
+      <c r="B23" s="157"/>
+      <c r="C23" s="149" t="s">
         <v>41</v>
       </c>
-      <c r="D23" s="142"/>
-      <c r="E23" s="133" t="s">
+      <c r="D23" s="150"/>
+      <c r="E23" s="141" t="s">
         <v>42</v>
       </c>
-      <c r="F23" s="134"/>
-      <c r="G23" s="143" t="s">
+      <c r="F23" s="142"/>
+      <c r="G23" s="151" t="s">
         <v>39</v>
       </c>
-      <c r="H23" s="144"/>
+      <c r="H23" s="152"/>
       <c r="I23" s="58"/>
-      <c r="J23" s="135" t="s">
+      <c r="J23" s="143" t="s">
         <v>43</v>
       </c>
-      <c r="K23" s="136"/>
-      <c r="L23" s="137" t="s">
+      <c r="K23" s="144"/>
+      <c r="L23" s="145" t="s">
         <v>44</v>
       </c>
-      <c r="M23" s="138"/>
-      <c r="N23" s="143" t="s">
+      <c r="M23" s="146"/>
+      <c r="N23" s="151" t="s">
         <v>40</v>
       </c>
-      <c r="O23" s="144"/>
+      <c r="O23" s="152"/>
       <c r="P23" s="58"/>
       <c r="Q23" s="68" t="s">
         <v>20</v>
@@ -5188,8 +5185,8 @@
       </c>
     </row>
     <row r="24" spans="1:18" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="150"/>
-      <c r="B24" s="150"/>
+      <c r="A24" s="158"/>
+      <c r="B24" s="158"/>
       <c r="C24" s="69" t="s">
         <v>22</v>
       </c>
@@ -5513,385 +5510,385 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="39.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="101" t="s">
+      <c r="A1" s="98" t="s">
         <v>71</v>
       </c>
-      <c r="B1" s="102" t="s">
+      <c r="B1" s="99" t="s">
         <v>72</v>
       </c>
-      <c r="C1" s="102" t="s">
+      <c r="C1" s="99" t="s">
         <v>73</v>
       </c>
-      <c r="D1" s="102" t="s">
+      <c r="D1" s="99" t="s">
         <v>74</v>
       </c>
-      <c r="E1" s="102" t="s">
+      <c r="E1" s="99" t="s">
         <v>75</v>
       </c>
-      <c r="F1" s="102" t="s">
+      <c r="F1" s="99" t="s">
         <v>76</v>
       </c>
-      <c r="G1" s="102" t="s">
+      <c r="G1" s="99" t="s">
         <v>77</v>
       </c>
-      <c r="H1" s="102" t="s">
+      <c r="H1" s="99" t="s">
         <v>78</v>
       </c>
-      <c r="I1" s="103" t="s">
+      <c r="I1" s="100" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="104"/>
-      <c r="B2" s="105"/>
-      <c r="C2" s="106"/>
-      <c r="D2" s="107"/>
-      <c r="E2" s="105"/>
-      <c r="F2" s="105"/>
-      <c r="G2" s="105"/>
-      <c r="H2" s="108"/>
-      <c r="I2" s="109"/>
+      <c r="A2" s="101"/>
+      <c r="B2" s="102"/>
+      <c r="C2" s="103"/>
+      <c r="D2" s="104"/>
+      <c r="E2" s="102"/>
+      <c r="F2" s="102"/>
+      <c r="G2" s="102"/>
+      <c r="H2" s="105"/>
+      <c r="I2" s="106"/>
     </row>
     <row r="3" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="110"/>
-      <c r="B3" s="111"/>
-      <c r="C3" s="112"/>
-      <c r="D3" s="113"/>
-      <c r="E3" s="111"/>
-      <c r="F3" s="111"/>
-      <c r="G3" s="111"/>
-      <c r="H3" s="114"/>
-      <c r="I3" s="115"/>
+      <c r="A3" s="107"/>
+      <c r="B3" s="108"/>
+      <c r="C3" s="109"/>
+      <c r="D3" s="110"/>
+      <c r="E3" s="108"/>
+      <c r="F3" s="108"/>
+      <c r="G3" s="108"/>
+      <c r="H3" s="111"/>
+      <c r="I3" s="112"/>
     </row>
     <row r="4" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="104"/>
-      <c r="B4" s="105"/>
-      <c r="C4" s="106"/>
-      <c r="D4" s="107"/>
-      <c r="E4" s="105"/>
-      <c r="F4" s="105"/>
-      <c r="G4" s="105"/>
-      <c r="H4" s="108"/>
-      <c r="I4" s="109"/>
+      <c r="A4" s="101"/>
+      <c r="B4" s="102"/>
+      <c r="C4" s="103"/>
+      <c r="D4" s="104"/>
+      <c r="E4" s="102"/>
+      <c r="F4" s="102"/>
+      <c r="G4" s="102"/>
+      <c r="H4" s="105"/>
+      <c r="I4" s="106"/>
     </row>
     <row r="5" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="110"/>
-      <c r="B5" s="111"/>
-      <c r="C5" s="112"/>
-      <c r="D5" s="113"/>
-      <c r="E5" s="111"/>
-      <c r="F5" s="111"/>
-      <c r="G5" s="111"/>
-      <c r="H5" s="114"/>
-      <c r="I5" s="115"/>
+      <c r="A5" s="107"/>
+      <c r="B5" s="108"/>
+      <c r="C5" s="109"/>
+      <c r="D5" s="110"/>
+      <c r="E5" s="108"/>
+      <c r="F5" s="108"/>
+      <c r="G5" s="108"/>
+      <c r="H5" s="111"/>
+      <c r="I5" s="112"/>
     </row>
     <row r="6" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="104"/>
-      <c r="B6" s="105"/>
-      <c r="C6" s="106"/>
-      <c r="D6" s="107"/>
-      <c r="E6" s="105"/>
-      <c r="F6" s="105"/>
-      <c r="G6" s="105"/>
-      <c r="H6" s="108"/>
-      <c r="I6" s="116"/>
+      <c r="A6" s="101"/>
+      <c r="B6" s="102"/>
+      <c r="C6" s="103"/>
+      <c r="D6" s="104"/>
+      <c r="E6" s="102"/>
+      <c r="F6" s="102"/>
+      <c r="G6" s="102"/>
+      <c r="H6" s="105"/>
+      <c r="I6" s="113"/>
     </row>
     <row r="7" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="110"/>
-      <c r="B7" s="111"/>
-      <c r="C7" s="112"/>
-      <c r="D7" s="113"/>
-      <c r="E7" s="111"/>
-      <c r="F7" s="111"/>
-      <c r="G7" s="111"/>
-      <c r="H7" s="114"/>
-      <c r="I7" s="117"/>
+      <c r="A7" s="107"/>
+      <c r="B7" s="108"/>
+      <c r="C7" s="109"/>
+      <c r="D7" s="110"/>
+      <c r="E7" s="108"/>
+      <c r="F7" s="108"/>
+      <c r="G7" s="108"/>
+      <c r="H7" s="111"/>
+      <c r="I7" s="114"/>
     </row>
     <row r="8" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="104"/>
-      <c r="B8" s="105"/>
-      <c r="C8" s="106"/>
-      <c r="D8" s="107"/>
-      <c r="E8" s="105"/>
-      <c r="F8" s="105"/>
-      <c r="G8" s="105"/>
-      <c r="H8" s="108"/>
-      <c r="I8" s="116"/>
+      <c r="A8" s="101"/>
+      <c r="B8" s="102"/>
+      <c r="C8" s="103"/>
+      <c r="D8" s="104"/>
+      <c r="E8" s="102"/>
+      <c r="F8" s="102"/>
+      <c r="G8" s="102"/>
+      <c r="H8" s="105"/>
+      <c r="I8" s="113"/>
     </row>
     <row r="9" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="110"/>
-      <c r="B9" s="111"/>
-      <c r="C9" s="112"/>
-      <c r="D9" s="113"/>
-      <c r="E9" s="111"/>
-      <c r="F9" s="111"/>
-      <c r="G9" s="111"/>
-      <c r="H9" s="114"/>
-      <c r="I9" s="118"/>
+      <c r="A9" s="107"/>
+      <c r="B9" s="108"/>
+      <c r="C9" s="109"/>
+      <c r="D9" s="110"/>
+      <c r="E9" s="108"/>
+      <c r="F9" s="108"/>
+      <c r="G9" s="108"/>
+      <c r="H9" s="111"/>
+      <c r="I9" s="115"/>
     </row>
     <row r="10" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="104"/>
-      <c r="B10" s="105"/>
-      <c r="C10" s="106"/>
-      <c r="D10" s="107"/>
-      <c r="E10" s="105"/>
-      <c r="F10" s="105"/>
-      <c r="G10" s="105"/>
-      <c r="H10" s="108"/>
-      <c r="I10" s="119"/>
+      <c r="A10" s="101"/>
+      <c r="B10" s="102"/>
+      <c r="C10" s="103"/>
+      <c r="D10" s="104"/>
+      <c r="E10" s="102"/>
+      <c r="F10" s="102"/>
+      <c r="G10" s="102"/>
+      <c r="H10" s="105"/>
+      <c r="I10" s="116"/>
     </row>
     <row r="11" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="110"/>
-      <c r="B11" s="111"/>
-      <c r="C11" s="112"/>
-      <c r="D11" s="113"/>
-      <c r="E11" s="111"/>
-      <c r="F11" s="111"/>
-      <c r="G11" s="111"/>
-      <c r="H11" s="114"/>
-      <c r="I11" s="120"/>
+      <c r="A11" s="107"/>
+      <c r="B11" s="108"/>
+      <c r="C11" s="109"/>
+      <c r="D11" s="110"/>
+      <c r="E11" s="108"/>
+      <c r="F11" s="108"/>
+      <c r="G11" s="108"/>
+      <c r="H11" s="111"/>
+      <c r="I11" s="117"/>
     </row>
     <row r="12" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="104"/>
-      <c r="B12" s="105"/>
-      <c r="C12" s="106"/>
-      <c r="D12" s="105"/>
-      <c r="E12" s="105"/>
-      <c r="F12" s="105"/>
-      <c r="G12" s="105"/>
-      <c r="H12" s="108"/>
-      <c r="I12" s="119"/>
+      <c r="A12" s="101"/>
+      <c r="B12" s="102"/>
+      <c r="C12" s="103"/>
+      <c r="D12" s="102"/>
+      <c r="E12" s="102"/>
+      <c r="F12" s="102"/>
+      <c r="G12" s="102"/>
+      <c r="H12" s="105"/>
+      <c r="I12" s="116"/>
     </row>
     <row r="13" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="110"/>
-      <c r="B13" s="111"/>
-      <c r="C13" s="112"/>
-      <c r="D13" s="111"/>
-      <c r="E13" s="111"/>
-      <c r="F13" s="111"/>
-      <c r="G13" s="111"/>
-      <c r="H13" s="114"/>
-      <c r="I13" s="120"/>
+      <c r="A13" s="107"/>
+      <c r="B13" s="108"/>
+      <c r="C13" s="109"/>
+      <c r="D13" s="108"/>
+      <c r="E13" s="108"/>
+      <c r="F13" s="108"/>
+      <c r="G13" s="108"/>
+      <c r="H13" s="111"/>
+      <c r="I13" s="117"/>
     </row>
     <row r="14" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="104"/>
-      <c r="B14" s="105"/>
-      <c r="C14" s="106"/>
-      <c r="D14" s="105"/>
-      <c r="E14" s="105"/>
-      <c r="F14" s="105"/>
-      <c r="G14" s="105"/>
-      <c r="H14" s="108"/>
-      <c r="I14" s="119"/>
+      <c r="A14" s="101"/>
+      <c r="B14" s="102"/>
+      <c r="C14" s="103"/>
+      <c r="D14" s="102"/>
+      <c r="E14" s="102"/>
+      <c r="F14" s="102"/>
+      <c r="G14" s="102"/>
+      <c r="H14" s="105"/>
+      <c r="I14" s="116"/>
     </row>
     <row r="15" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="110"/>
-      <c r="B15" s="111"/>
-      <c r="C15" s="112"/>
-      <c r="D15" s="111"/>
-      <c r="E15" s="111"/>
-      <c r="F15" s="111"/>
-      <c r="G15" s="111"/>
-      <c r="H15" s="114"/>
-      <c r="I15" s="120"/>
+      <c r="A15" s="107"/>
+      <c r="B15" s="108"/>
+      <c r="C15" s="109"/>
+      <c r="D15" s="108"/>
+      <c r="E15" s="108"/>
+      <c r="F15" s="108"/>
+      <c r="G15" s="108"/>
+      <c r="H15" s="111"/>
+      <c r="I15" s="117"/>
     </row>
     <row r="16" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="104"/>
-      <c r="B16" s="105"/>
-      <c r="C16" s="106"/>
-      <c r="D16" s="105"/>
-      <c r="E16" s="105"/>
-      <c r="F16" s="105"/>
-      <c r="G16" s="105"/>
-      <c r="H16" s="108"/>
-      <c r="I16" s="119"/>
+      <c r="A16" s="101"/>
+      <c r="B16" s="102"/>
+      <c r="C16" s="103"/>
+      <c r="D16" s="102"/>
+      <c r="E16" s="102"/>
+      <c r="F16" s="102"/>
+      <c r="G16" s="102"/>
+      <c r="H16" s="105"/>
+      <c r="I16" s="116"/>
     </row>
     <row r="17" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="110"/>
-      <c r="B17" s="111"/>
-      <c r="C17" s="112"/>
-      <c r="D17" s="113"/>
-      <c r="E17" s="111"/>
-      <c r="F17" s="111"/>
-      <c r="G17" s="111"/>
-      <c r="H17" s="114"/>
-      <c r="I17" s="120"/>
+      <c r="A17" s="107"/>
+      <c r="B17" s="108"/>
+      <c r="C17" s="109"/>
+      <c r="D17" s="110"/>
+      <c r="E17" s="108"/>
+      <c r="F17" s="108"/>
+      <c r="G17" s="108"/>
+      <c r="H17" s="111"/>
+      <c r="I17" s="117"/>
     </row>
     <row r="18" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="104"/>
-      <c r="B18" s="105"/>
-      <c r="C18" s="105"/>
-      <c r="D18" s="105"/>
-      <c r="E18" s="105"/>
-      <c r="F18" s="105"/>
-      <c r="G18" s="105"/>
-      <c r="H18" s="108"/>
-      <c r="I18" s="109"/>
+      <c r="A18" s="101"/>
+      <c r="B18" s="102"/>
+      <c r="C18" s="102"/>
+      <c r="D18" s="102"/>
+      <c r="E18" s="102"/>
+      <c r="F18" s="102"/>
+      <c r="G18" s="102"/>
+      <c r="H18" s="105"/>
+      <c r="I18" s="106"/>
     </row>
     <row r="19" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="110"/>
-      <c r="B19" s="111"/>
-      <c r="C19" s="112"/>
-      <c r="D19" s="111"/>
-      <c r="E19" s="111"/>
-      <c r="F19" s="111"/>
-      <c r="G19" s="111"/>
-      <c r="H19" s="114"/>
-      <c r="I19" s="120"/>
+      <c r="A19" s="107"/>
+      <c r="B19" s="108"/>
+      <c r="C19" s="109"/>
+      <c r="D19" s="108"/>
+      <c r="E19" s="108"/>
+      <c r="F19" s="108"/>
+      <c r="G19" s="108"/>
+      <c r="H19" s="111"/>
+      <c r="I19" s="117"/>
     </row>
     <row r="20" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="104"/>
-      <c r="B20" s="105"/>
-      <c r="C20" s="106"/>
-      <c r="D20" s="105"/>
-      <c r="E20" s="105"/>
-      <c r="F20" s="105"/>
-      <c r="G20" s="105"/>
-      <c r="H20" s="108"/>
-      <c r="I20" s="119"/>
+      <c r="A20" s="101"/>
+      <c r="B20" s="102"/>
+      <c r="C20" s="103"/>
+      <c r="D20" s="102"/>
+      <c r="E20" s="102"/>
+      <c r="F20" s="102"/>
+      <c r="G20" s="102"/>
+      <c r="H20" s="105"/>
+      <c r="I20" s="116"/>
     </row>
     <row r="21" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="110"/>
-      <c r="B21" s="111"/>
-      <c r="C21" s="112"/>
-      <c r="D21" s="111"/>
-      <c r="E21" s="111"/>
-      <c r="F21" s="111"/>
-      <c r="G21" s="111"/>
-      <c r="H21" s="114"/>
-      <c r="I21" s="120"/>
+      <c r="A21" s="107"/>
+      <c r="B21" s="108"/>
+      <c r="C21" s="109"/>
+      <c r="D21" s="108"/>
+      <c r="E21" s="108"/>
+      <c r="F21" s="108"/>
+      <c r="G21" s="108"/>
+      <c r="H21" s="111"/>
+      <c r="I21" s="117"/>
     </row>
     <row r="22" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="104"/>
-      <c r="B22" s="105"/>
-      <c r="C22" s="106"/>
-      <c r="D22" s="105"/>
-      <c r="E22" s="105"/>
-      <c r="F22" s="105"/>
-      <c r="G22" s="105"/>
-      <c r="H22" s="108"/>
-      <c r="I22" s="116"/>
+      <c r="A22" s="101"/>
+      <c r="B22" s="102"/>
+      <c r="C22" s="103"/>
+      <c r="D22" s="102"/>
+      <c r="E22" s="102"/>
+      <c r="F22" s="102"/>
+      <c r="G22" s="102"/>
+      <c r="H22" s="105"/>
+      <c r="I22" s="113"/>
     </row>
     <row r="23" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="110"/>
-      <c r="B23" s="111"/>
-      <c r="C23" s="112"/>
-      <c r="D23" s="111"/>
-      <c r="E23" s="111"/>
-      <c r="F23" s="111"/>
-      <c r="G23" s="111"/>
-      <c r="H23" s="114"/>
-      <c r="I23" s="117"/>
+      <c r="A23" s="107"/>
+      <c r="B23" s="108"/>
+      <c r="C23" s="109"/>
+      <c r="D23" s="108"/>
+      <c r="E23" s="108"/>
+      <c r="F23" s="108"/>
+      <c r="G23" s="108"/>
+      <c r="H23" s="111"/>
+      <c r="I23" s="114"/>
     </row>
     <row r="24" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="104"/>
-      <c r="B24" s="105"/>
-      <c r="C24" s="106"/>
-      <c r="D24" s="105"/>
-      <c r="E24" s="105"/>
-      <c r="F24" s="105"/>
-      <c r="G24" s="105"/>
-      <c r="H24" s="108"/>
-      <c r="I24" s="116"/>
+      <c r="A24" s="101"/>
+      <c r="B24" s="102"/>
+      <c r="C24" s="103"/>
+      <c r="D24" s="102"/>
+      <c r="E24" s="102"/>
+      <c r="F24" s="102"/>
+      <c r="G24" s="102"/>
+      <c r="H24" s="105"/>
+      <c r="I24" s="113"/>
     </row>
     <row r="25" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="110"/>
-      <c r="B25" s="111"/>
-      <c r="C25" s="112"/>
-      <c r="D25" s="111"/>
-      <c r="E25" s="111"/>
-      <c r="F25" s="111"/>
-      <c r="G25" s="111"/>
-      <c r="H25" s="114"/>
-      <c r="I25" s="117"/>
+      <c r="A25" s="107"/>
+      <c r="B25" s="108"/>
+      <c r="C25" s="109"/>
+      <c r="D25" s="108"/>
+      <c r="E25" s="108"/>
+      <c r="F25" s="108"/>
+      <c r="G25" s="108"/>
+      <c r="H25" s="111"/>
+      <c r="I25" s="114"/>
     </row>
     <row r="26" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="104"/>
-      <c r="B26" s="105"/>
-      <c r="C26" s="106"/>
-      <c r="D26" s="105"/>
-      <c r="E26" s="105"/>
-      <c r="F26" s="105"/>
-      <c r="G26" s="105"/>
-      <c r="H26" s="108"/>
-      <c r="I26" s="116"/>
+      <c r="A26" s="101"/>
+      <c r="B26" s="102"/>
+      <c r="C26" s="103"/>
+      <c r="D26" s="102"/>
+      <c r="E26" s="102"/>
+      <c r="F26" s="102"/>
+      <c r="G26" s="102"/>
+      <c r="H26" s="105"/>
+      <c r="I26" s="113"/>
     </row>
     <row r="27" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="110"/>
-      <c r="B27" s="111"/>
-      <c r="C27" s="112"/>
-      <c r="D27" s="111"/>
-      <c r="E27" s="111"/>
-      <c r="F27" s="111"/>
-      <c r="G27" s="111"/>
-      <c r="H27" s="114"/>
-      <c r="I27" s="117"/>
+      <c r="A27" s="107"/>
+      <c r="B27" s="108"/>
+      <c r="C27" s="109"/>
+      <c r="D27" s="108"/>
+      <c r="E27" s="108"/>
+      <c r="F27" s="108"/>
+      <c r="G27" s="108"/>
+      <c r="H27" s="111"/>
+      <c r="I27" s="114"/>
     </row>
     <row r="28" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="104"/>
-      <c r="B28" s="105"/>
-      <c r="C28" s="106"/>
-      <c r="D28" s="105"/>
-      <c r="E28" s="105"/>
-      <c r="F28" s="105"/>
-      <c r="G28" s="105"/>
-      <c r="H28" s="108"/>
-      <c r="I28" s="116"/>
+      <c r="A28" s="101"/>
+      <c r="B28" s="102"/>
+      <c r="C28" s="103"/>
+      <c r="D28" s="102"/>
+      <c r="E28" s="102"/>
+      <c r="F28" s="102"/>
+      <c r="G28" s="102"/>
+      <c r="H28" s="105"/>
+      <c r="I28" s="113"/>
     </row>
     <row r="29" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="110"/>
-      <c r="B29" s="111"/>
-      <c r="C29" s="112"/>
-      <c r="D29" s="111"/>
-      <c r="E29" s="111"/>
-      <c r="F29" s="111"/>
-      <c r="G29" s="111"/>
-      <c r="H29" s="114"/>
-      <c r="I29" s="117"/>
+      <c r="A29" s="107"/>
+      <c r="B29" s="108"/>
+      <c r="C29" s="109"/>
+      <c r="D29" s="108"/>
+      <c r="E29" s="108"/>
+      <c r="F29" s="108"/>
+      <c r="G29" s="108"/>
+      <c r="H29" s="111"/>
+      <c r="I29" s="114"/>
     </row>
     <row r="30" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="104"/>
-      <c r="B30" s="105"/>
-      <c r="C30" s="106"/>
-      <c r="D30" s="105"/>
-      <c r="E30" s="105"/>
-      <c r="F30" s="105"/>
-      <c r="G30" s="105"/>
-      <c r="H30" s="108"/>
-      <c r="I30" s="116"/>
+      <c r="A30" s="101"/>
+      <c r="B30" s="102"/>
+      <c r="C30" s="103"/>
+      <c r="D30" s="102"/>
+      <c r="E30" s="102"/>
+      <c r="F30" s="102"/>
+      <c r="G30" s="102"/>
+      <c r="H30" s="105"/>
+      <c r="I30" s="113"/>
     </row>
     <row r="31" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="110"/>
-      <c r="B31" s="111"/>
-      <c r="C31" s="112"/>
-      <c r="D31" s="111"/>
-      <c r="E31" s="111"/>
-      <c r="F31" s="111"/>
-      <c r="G31" s="111"/>
-      <c r="H31" s="114"/>
-      <c r="I31" s="117"/>
+      <c r="A31" s="107"/>
+      <c r="B31" s="108"/>
+      <c r="C31" s="109"/>
+      <c r="D31" s="108"/>
+      <c r="E31" s="108"/>
+      <c r="F31" s="108"/>
+      <c r="G31" s="108"/>
+      <c r="H31" s="111"/>
+      <c r="I31" s="114"/>
     </row>
     <row r="32" spans="1:9" ht="20.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="104"/>
-      <c r="B32" s="105"/>
-      <c r="C32" s="106"/>
-      <c r="D32" s="105"/>
-      <c r="E32" s="105"/>
-      <c r="F32" s="105"/>
-      <c r="G32" s="105"/>
-      <c r="H32" s="121"/>
-      <c r="I32" s="116"/>
+      <c r="A32" s="101"/>
+      <c r="B32" s="102"/>
+      <c r="C32" s="103"/>
+      <c r="D32" s="102"/>
+      <c r="E32" s="102"/>
+      <c r="F32" s="102"/>
+      <c r="G32" s="102"/>
+      <c r="H32" s="118"/>
+      <c r="I32" s="113"/>
     </row>
     <row r="33" spans="1:9" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="122"/>
-      <c r="B33" s="123"/>
-      <c r="C33" s="123"/>
-      <c r="D33" s="123"/>
-      <c r="E33" s="123"/>
-      <c r="F33" s="123"/>
-      <c r="G33" s="123"/>
-      <c r="H33" s="123"/>
-      <c r="I33" s="118"/>
+      <c r="A33" s="119"/>
+      <c r="B33" s="120"/>
+      <c r="C33" s="120"/>
+      <c r="D33" s="120"/>
+      <c r="E33" s="120"/>
+      <c r="F33" s="120"/>
+      <c r="G33" s="120"/>
+      <c r="H33" s="120"/>
+      <c r="I33" s="115"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>